<commit_message>
Synchronize validated research beta snapshot
</commit_message>
<xml_diff>
--- a/research-beta/outputs/branch-registry/Welsh-LDS-Branch-Registry.xlsx
+++ b/research-beta/outputs/branch-registry/Welsh-LDS-Branch-Registry.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Registry" sheetId="1" r:id="Rd20d70fb12bc40ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="Rfff5572052eb4646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R9bad88b556964fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Registry" sheetId="1" r:id="R961ccdbd956446af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Log" sheetId="2" r:id="R12f68d3ff0794e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="Rc55590f7cc7e4d7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -151,12 +151,12 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{E6BDC08C-84FE-4C36-8721-BEE5861C26C6}"/>
+  <xltc:person displayName="User" id="{E67A5C1B-06C4-4D29-BF93-B4F2DE95DFCC}"/>
 </xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BranchRegistryTable" displayName="BranchRegistryTable" ref="A1:N61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BranchRegistryTable" displayName="BranchRegistryTable" ref="A1:N62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Canonical name"/>
     <x:tableColumn id="2" name="Entity type"/>
@@ -178,7 +178,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BranchEvidenceTable" displayName="BranchEvidenceTable" ref="A1:I140" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BranchEvidenceTable" displayName="BranchEvidenceTable" ref="A1:I160" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Raw name as found"/>
     <x:tableColumn id="2" name="Proposed canonical name"/>
@@ -922,7 +922,7 @@
         <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J14" s="5" t="str">
-        <x:v>Wales2Utah research note; Film 104168 Item 10</x:v>
+        <x:v>Photographed library identifier 859; four bounded register frames within a nine-frame compound packet; Wales2Utah research note; Film 104168 Item 10</x:v>
       </x:c>
       <x:c r="K14" s="5" t="str"/>
       <x:c r="L14" s="5" t="str"/>
@@ -1058,7 +1058,7 @@
         <x:v>1874</x:v>
       </x:c>
       <x:c r="F18" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G18" s="4" t="str">
         <x:v>No</x:v>
@@ -1067,15 +1067,15 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I18" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Contextual typed minutes evidence; dedicated member register not recovered</x:v>
       </x:c>
       <x:c r="J18" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
+        <x:v>CD 62 within source group CDs 60-62; LR 70861 1; Pontypool/Abersychan General Minutes, 1857-1889; Cwmbran reports on typed PDF pages 129, 167, 169, 171-172, 176; Film 104168 Item 13 retained as legacy discovery metadata</x:v>
       </x:c>
       <x:c r="K18" s="5" t="str"/>
       <x:c r="L18" s="5" t="str"/>
       <x:c r="M18" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+        <x:v>Cwmbran is repeatedly attested in branch-condition, missionary, baptism/addition, and appointment reports. This is contextual minutes evidence, not a dedicated Record of Members.</x:v>
       </x:c>
       <x:c r="N18" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
@@ -1108,7 +1108,7 @@
         <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J19" s="5" t="str">
-        <x:v>Film 104168 Item 12</x:v>
+        <x:v>Film 104168 Item 12; no matching local image or PDF packet located; Film 104168 Item 12</x:v>
       </x:c>
       <x:c r="K19" s="5" t="str"/>
       <x:c r="L19" s="5" t="str"/>
@@ -1133,7 +1133,7 @@
         <x:v>1847</x:v>
       </x:c>
       <x:c r="E20" s="6" t="n">
-        <x:v>1862</x:v>
+        <x:v>1857</x:v>
       </x:c>
       <x:c r="F20" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1148,7 +1148,7 @@
         <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J20" s="5" t="str">
-        <x:v>CD 8; LR 188 7; Wales2Utah research note</x:v>
+        <x:v>CD 8; LR 188 7; CD 8; LR 188 7; photographed library identifier 859; 69 authoritative full-resolution images; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K20" s="5" t="str"/>
       <x:c r="L20" s="5" t="str"/>
@@ -1305,52 +1305,60 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="4" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="B25" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C25" s="5" t="str">
-        <x:v>Festiniog</x:v>
+        <x:v>Eglwys Fach; Eglwys Bach</x:v>
       </x:c>
       <x:c r="D25" s="6" t="n">
-        <x:v>1848</x:v>
+        <x:v>1849</x:v>
       </x:c>
       <x:c r="E25" s="6" t="n">
-        <x:v>1856</x:v>
+        <x:v>1864</x:v>
       </x:c>
       <x:c r="F25" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G25" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H25" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I25" s="5" t="str">
-        <x:v>Research note only</x:v>
+        <x:v>Historically verified branch; recorded branch book not currently located</x:v>
       </x:c>
       <x:c r="J25" s="5" t="str">
-        <x:v>Ffestiniog membership record book integrated into local archive; surviving title uses Festiniog; 94 unique viewer images; Wales2Utah research note</x:v>
+        <x:v>Abel Evans organized a six-member branch; Hugh Roberts served as presiding elder and kept the branch record until emigrating in 1864; Historical/source spelling used in Hugh Roberts family records; Variant spacing retained for discovery; Conwy Valley Conference held at Eglwysbach, 28 May 1854; five branches and 98 members reported for the conference</x:v>
       </x:c>
       <x:c r="K25" s="5" t="str"/>
       <x:c r="L25" s="5" t="str"/>
       <x:c r="M25" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N25" s="5" t="str"/>
+        <x:v>Organized by Abel Evans with six members after the Roberts family conversions; Hugh Roberts served as presiding elder and kept the branch record until 1864. The record's present survival or location is unknown.</x:v>
+      </x:c>
+      <x:c r="N25" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Immigrant_View.aspx?id=806</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="4" t="str">
-        <x:v>Georgetown</x:v>
+        <x:v>Ffestiniog</x:v>
       </x:c>
       <x:c r="B26" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C26" s="5" t="str"/>
-      <x:c r="D26" s="6"/>
-      <x:c r="E26" s="6"/>
+      <x:c r="C26" s="5" t="str">
+        <x:v>Festiniog</x:v>
+      </x:c>
+      <x:c r="D26" s="6" t="n">
+        <x:v>1848</x:v>
+      </x:c>
+      <x:c r="E26" s="6" t="n">
+        <x:v>1856</x:v>
+      </x:c>
       <x:c r="F26" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -1364,7 +1372,7 @@
         <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J26" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>Ffestiniog membership record book integrated into local archive; surviving title uses Festiniog; 94 unique viewer images; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K26" s="5" t="str"/>
       <x:c r="L26" s="5" t="str"/>
@@ -1375,20 +1383,16 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="4" t="str">
-        <x:v>Gilwern</x:v>
+        <x:v>Georgetown</x:v>
       </x:c>
       <x:c r="B27" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str"/>
-      <x:c r="D27" s="6" t="n">
-        <x:v>1849</x:v>
-      </x:c>
-      <x:c r="E27" s="6" t="n">
-        <x:v>1858</x:v>
-      </x:c>
+      <x:c r="D27" s="6"/>
+      <x:c r="E27" s="6"/>
       <x:c r="F27" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G27" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1397,10 +1401,10 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I27" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J27" s="5" t="str">
-        <x:v>CD 7; LR 13987 7; Wales2Utah research note</x:v>
+        <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K27" s="5" t="str"/>
       <x:c r="L27" s="5" t="str"/>
@@ -1411,17 +1415,17 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="4" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Gilwern</x:v>
       </x:c>
       <x:c r="B28" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str"/>
       <x:c r="D28" s="6" t="n">
-        <x:v>1847</x:v>
+        <x:v>1849</x:v>
       </x:c>
       <x:c r="E28" s="6" t="n">
-        <x:v>1860</x:v>
+        <x:v>1858</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1433,29 +1437,31 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I28" s="5" t="str">
-        <x:v>Verified local source collection</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J28" s="5" t="str">
-        <x:v>CD 23 / CR 11343 11 V.1; CD 58 / CR 11343 11 V.2; 272 authoritative historical images; membership registers 1847-1853 and 1857-1860</x:v>
+        <x:v>CD 7; LR 13987 7; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K28" s="5" t="str"/>
       <x:c r="L28" s="5" t="str"/>
-      <x:c r="M28" s="5" t="str"/>
+      <x:c r="M28" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
       <x:c r="N28" s="5" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="4" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="B29" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str"/>
       <x:c r="D29" s="6" t="n">
-        <x:v>1849</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="E29" s="6" t="n">
-        <x:v>1866</x:v>
+        <x:v>1860</x:v>
       </x:c>
       <x:c r="F29" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1470,7 +1476,7 @@
         <x:v>Verified local source collection</x:v>
       </x:c>
       <x:c r="J29" s="5" t="str">
-        <x:v>CD 22; project LR 113 7; photographed library identifier 870 preserved separately; 45 authoritative full-resolution images; source dates 1849-1866</x:v>
+        <x:v>CD 23 / CR 11343 11 V.1; CD 58 / CR 11343 11 V.2; 272 authoritative historical images; membership registers 1847-1853 and 1857-1860</x:v>
       </x:c>
       <x:c r="K29" s="5" t="str"/>
       <x:c r="L29" s="5" t="str"/>
@@ -1479,19 +1485,17 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="4" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="B30" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C30" s="5" t="str">
-        <x:v>Llanelly</x:v>
-      </x:c>
+      <x:c r="C30" s="5" t="str"/>
       <x:c r="D30" s="6" t="n">
-        <x:v>1847</x:v>
+        <x:v>1849</x:v>
       </x:c>
       <x:c r="E30" s="6" t="n">
-        <x:v>1868</x:v>
+        <x:v>1866</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1503,33 +1507,31 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I30" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Verified local source collection</x:v>
       </x:c>
       <x:c r="J30" s="5" t="str">
-        <x:v>CD 11; LR 11757 7; CD 11; source label 1577; recovered folder LR 11757 7; filename prefix LR 12451 7 (unresolved conflict); Wales2Utah research note</x:v>
+        <x:v>CD 22; project LR 113 7; photographed library identifier 870 preserved separately; 45 authoritative full-resolution images; source dates 1849-1866</x:v>
       </x:c>
       <x:c r="K30" s="5" t="str"/>
       <x:c r="L30" s="5" t="str"/>
-      <x:c r="M30" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M30" s="5" t="str"/>
       <x:c r="N30" s="5" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="4" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="B31" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
-        <x:v>Llanellyd; Llanelltud</x:v>
+        <x:v>Llanelly</x:v>
       </x:c>
       <x:c r="D31" s="6" t="n">
-        <x:v>1850</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="E31" s="6" t="n">
-        <x:v>1857</x:v>
+        <x:v>1868</x:v>
       </x:c>
       <x:c r="F31" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1538,69 +1540,71 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H31" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I31" s="5" t="str">
-        <x:v>Verified compound local source section</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J31" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound section; internal pages 1-5; 10 authoritative full-resolution images; section dated 1850-1857</x:v>
+        <x:v>CD 11; LR 11757 7; CD 11; source label 1577; recovered folder LR 11757 7; filename prefix LR 12451 7 (unresolved conflict); Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K31" s="5" t="str"/>
       <x:c r="L31" s="5" t="str"/>
-      <x:c r="M31" s="5" t="str"/>
-      <x:c r="N31" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
+      <x:c r="M31" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N31" s="5" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="4" t="str">
-        <x:v>Llanelly 2</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="B32" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C32" s="5" t="str"/>
-      <x:c r="D32" s="6"/>
-      <x:c r="E32" s="6"/>
+      <x:c r="C32" s="5" t="str">
+        <x:v>Llanellyd; Llanelltud</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="n">
+        <x:v>1850</x:v>
+      </x:c>
+      <x:c r="E32" s="6" t="n">
+        <x:v>1857</x:v>
+      </x:c>
       <x:c r="F32" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G32" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H32" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="I32" s="5" t="str">
-        <x:v>Research note only</x:v>
+        <x:v>Verified compound local source section</x:v>
       </x:c>
       <x:c r="J32" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 34; LR 172 7 compound section; internal pages 1-5; 10 authoritative full-resolution images; section dated 1850-1857</x:v>
       </x:c>
       <x:c r="K32" s="5" t="str"/>
       <x:c r="L32" s="5" t="str"/>
-      <x:c r="M32" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N32" s="5" t="str"/>
+      <x:c r="M32" s="5" t="str"/>
+      <x:c r="N32" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="4" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Llanelly 2</x:v>
       </x:c>
       <x:c r="B33" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C33" s="5" t="str"/>
-      <x:c r="D33" s="6" t="n">
-        <x:v>1847</x:v>
-      </x:c>
-      <x:c r="E33" s="6" t="n">
-        <x:v>1869</x:v>
-      </x:c>
+      <x:c r="D33" s="6"/>
+      <x:c r="E33" s="6"/>
       <x:c r="F33" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G33" s="4" t="str">
         <x:v>Yes</x:v>
@@ -1609,53 +1613,51 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I33" s="5" t="str">
-        <x:v>Verified local source collection</x:v>
+        <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J33" s="5" t="str">
-        <x:v>CD 15; project LR1687; historical/library identifier 871 preserved separately; 60 authoritative full-resolution images</x:v>
+        <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K33" s="5" t="str"/>
       <x:c r="L33" s="5" t="str"/>
-      <x:c r="M33" s="5" t="str"/>
+      <x:c r="M33" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
       <x:c r="N33" s="5" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="4" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="B34" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str"/>
       <x:c r="D34" s="6" t="n">
-        <x:v>1849</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="E34" s="6" t="n">
-        <x:v>1879</x:v>
+        <x:v>1869</x:v>
       </x:c>
       <x:c r="F34" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G34" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H34" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I34" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Verified local source collection</x:v>
       </x:c>
       <x:c r="J34" s="5" t="str">
-        <x:v>Wales2Utah research note; Film 104169 items 14-15</x:v>
+        <x:v>CD 15; project LR1687; historical/library identifier 871 preserved separately; 60 authoritative full-resolution images</x:v>
       </x:c>
       <x:c r="K34" s="5" t="str"/>
       <x:c r="L34" s="5" t="str"/>
-      <x:c r="M34" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N34" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
-      </x:c>
+      <x:c r="M34" s="5" t="str"/>
+      <x:c r="N34" s="5" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="4" t="str">
@@ -1664,7 +1666,9 @@
       <x:c r="B35" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C35" s="5" t="str"/>
+      <x:c r="C35" s="5" t="str">
+        <x:v>Llansawel</x:v>
+      </x:c>
       <x:c r="D35" s="6" t="n">
         <x:v>1849</x:v>
       </x:c>
@@ -1681,17 +1685,17 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I35" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Verified dedicated local source collection</x:v>
       </x:c>
       <x:c r="J35" s="5" t="str">
-        <x:v>CD 14; LR 221 7</x:v>
+        <x:v>CD 14; LR 221 7; CD 14; LR 221 7; photographed library identifier 318; 28 authoritative images; Film 104169 items 14-15; locality assignment requires the recovered CD 14 source</x:v>
       </x:c>
       <x:c r="K35" s="5" t="str"/>
       <x:c r="L35" s="5" t="str"/>
-      <x:c r="M35" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N35" s="5" t="str"/>
+      <x:c r="M35" s="5" t="str"/>
+      <x:c r="N35" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="4" t="str">
@@ -1700,7 +1704,9 @@
       <x:c r="B36" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C36" s="5" t="str"/>
+      <x:c r="C36" s="5" t="str">
+        <x:v>Llansawel</x:v>
+      </x:c>
       <x:c r="D36" s="6" t="n">
         <x:v>1850</x:v>
       </x:c>
@@ -1717,17 +1723,17 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I36" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Verified compound local source section</x:v>
       </x:c>
       <x:c r="J36" s="5" t="str">
-        <x:v>CD 18; LR 11759 7</x:v>
+        <x:v>CD 18; LR 11759 7; CD 18; LR 11759 7; explicit images 00009-00048; 40 authoritative in-place images; Film 104169 items 14-15; locality assignment requires the recovered LR 11759 7 heading</x:v>
       </x:c>
       <x:c r="K36" s="5" t="str"/>
       <x:c r="L36" s="5" t="str"/>
-      <x:c r="M36" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N36" s="5" t="str"/>
+      <x:c r="M36" s="5" t="str"/>
+      <x:c r="N36" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="4" t="str">
@@ -1756,7 +1762,7 @@
         <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J37" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>18 recovered PDF frames; photographed identifier unresolved as 1565 versus 1765; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K37" s="5" t="str"/>
       <x:c r="L37" s="5" t="str"/>
@@ -1816,7 +1822,7 @@
         <x:v>1868</x:v>
       </x:c>
       <x:c r="F39" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G39" s="4" t="str">
         <x:v>No</x:v>
@@ -1825,15 +1831,15 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I39" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Contextual conference-minutes evidence; dedicated member register not recovered</x:v>
       </x:c>
       <x:c r="J39" s="5" t="str">
-        <x:v>Film 104172 Item 5</x:v>
+        <x:v>CD 41; LR 17617 21; Western Glamorgan Conference Minutes, 1851-1870; Morriston fast-offerings report, 1866; Film 104172 Item 5 retained as legacy discovery metadata</x:v>
       </x:c>
       <x:c r="K39" s="5" t="str"/>
       <x:c r="L39" s="5" t="str"/>
       <x:c r="M39" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+        <x:v>Morriston is explicitly attested by a 1866 fast-offerings report in the enclosing conference minutes. This is contextual conference material, not a dedicated Record of Members.</x:v>
       </x:c>
       <x:c r="N39" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
@@ -1915,57 +1921,65 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="4" t="str">
-        <x:v>Pen-y-cae</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="B42" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str">
-        <x:v>Pen-Y-Cae</x:v>
+        <x:v>Owrtyn</x:v>
       </x:c>
       <x:c r="D42" s="6" t="n">
-        <x:v>1844</x:v>
+        <x:v>1840</x:v>
       </x:c>
       <x:c r="E42" s="6" t="n">
-        <x:v>1866</x:v>
+        <x:v>1842</x:v>
       </x:c>
       <x:c r="F42" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G42" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H42" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I42" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Historically verified branch; no surviving local membership register identified</x:v>
       </x:c>
       <x:c r="J42" s="5" t="str">
-        <x:v>CD 17; LR 230 7; Wales2Utah research note</x:v>
+        <x:v>Overton: The First LDS Branch in Wales; organized 30 October 1840; earliest documented branch in Wales; Welsh spelling used in Welsh Saints person records for Overton, Flintshire; Opposition to the Gospel Message in Wales, PDF page 23; missionaries arrived 16 October and organized a branch 30 October 1840</x:v>
       </x:c>
       <x:c r="K42" s="5" t="str"/>
       <x:c r="L42" s="5" t="str"/>
       <x:c r="M42" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N42" s="5" t="str"/>
+        <x:v>Organized 30 October 1840 and documented as the first branch in Wales. Activity is documented through 1842; no surviving Overton membership register is currently identified.</x:v>
+      </x:c>
+      <x:c r="N42" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Resource_Info.aspx?id=24497</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="4" t="str">
-        <x:v>Pen-y-Darran</x:v>
+        <x:v>Pen-y-cae</x:v>
       </x:c>
       <x:c r="B43" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C43" s="5" t="str"/>
-      <x:c r="D43" s="6"/>
-      <x:c r="E43" s="6"/>
+      <x:c r="C43" s="5" t="str">
+        <x:v>Pen-Y-Cae</x:v>
+      </x:c>
+      <x:c r="D43" s="6" t="n">
+        <x:v>1844</x:v>
+      </x:c>
+      <x:c r="E43" s="6" t="n">
+        <x:v>1866</x:v>
+      </x:c>
       <x:c r="F43" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G43" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H43" s="4" t="str">
         <x:v>No</x:v>
@@ -1974,7 +1988,7 @@
         <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J43" s="5" t="str">
-        <x:v>CD 36; two-page baptism list</x:v>
+        <x:v>CD 17; LR 230 7; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K43" s="5" t="str"/>
       <x:c r="L43" s="5" t="str"/>
@@ -1985,22 +1999,16 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="4" t="str">
-        <x:v>Pendoylon</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="B44" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C44" s="5" t="str">
-        <x:v>Pendoylan</x:v>
-      </x:c>
-      <x:c r="D44" s="6" t="n">
-        <x:v>1851</x:v>
-      </x:c>
-      <x:c r="E44" s="6" t="n">
-        <x:v>1886</x:v>
-      </x:c>
+      <x:c r="C44" s="5" t="str"/>
+      <x:c r="D44" s="6"/>
+      <x:c r="E44" s="6"/>
       <x:c r="F44" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G44" s="4" t="str">
         <x:v>No</x:v>
@@ -2009,80 +2017,82 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="I44" s="5" t="str">
-        <x:v>Historical source attestation; local image collection not yet located</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J44" s="5" t="str">
-        <x:v>DGS 106248102; indexing images 195-239; WALES (Country), Part 5; Historical/source spelling in typed Cardiff conference records</x:v>
+        <x:v>CD 36; two-page baptism list</x:v>
       </x:c>
       <x:c r="K44" s="5" t="str"/>
       <x:c r="L44" s="5" t="str"/>
-      <x:c r="M44" s="5" t="str"/>
+      <x:c r="M44" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
       <x:c r="N44" s="5" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="4" t="str">
-        <x:v>Pontlanfraith</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="B45" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C45" s="5" t="str"/>
+      <x:c r="C45" s="5" t="str">
+        <x:v>Pendoylan</x:v>
+      </x:c>
       <x:c r="D45" s="6" t="n">
-        <x:v>1947</x:v>
+        <x:v>1851</x:v>
       </x:c>
       <x:c r="E45" s="6" t="n">
-        <x:v>1947</x:v>
+        <x:v>1886</x:v>
       </x:c>
       <x:c r="F45" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G45" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H45" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I45" s="5" t="str">
-        <x:v>Research note only</x:v>
+        <x:v>Historical source attestation; local image collection not yet located</x:v>
       </x:c>
       <x:c r="J45" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>DGS 106248102; indexing images 195-239; no matching local image or PDF packet located; DGS 106248102; indexing images 195-239; WALES (Country), Part 5; Historical/source spelling in typed Cardiff conference records</x:v>
       </x:c>
       <x:c r="K45" s="5" t="str"/>
       <x:c r="L45" s="5" t="str"/>
-      <x:c r="M45" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M45" s="5" t="str"/>
       <x:c r="N45" s="5" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="4" t="str">
-        <x:v>Pontypool</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="B46" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str"/>
       <x:c r="D46" s="6" t="n">
-        <x:v>1857</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="E46" s="6" t="n">
-        <x:v>1884</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="F46" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G46" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H46" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I46" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J46" s="5" t="str">
-        <x:v>CD 62; general minutes</x:v>
+        <x:v>10-page source packet; photographed library identifier 27560; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K46" s="5" t="str"/>
       <x:c r="L46" s="5" t="str"/>
@@ -2093,32 +2103,32 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="4" t="str">
-        <x:v>Pontypridd</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="B47" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str"/>
       <x:c r="D47" s="6" t="n">
-        <x:v>1877</x:v>
+        <x:v>1857</x:v>
       </x:c>
       <x:c r="E47" s="6" t="n">
-        <x:v>1895</x:v>
+        <x:v>1884</x:v>
       </x:c>
       <x:c r="F47" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G47" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H47" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I47" s="5" t="str">
-        <x:v>Research note only</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J47" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="K47" s="5" t="str"/>
       <x:c r="L47" s="5" t="str"/>
@@ -2129,32 +2139,32 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="4" t="str">
-        <x:v>Rhymney</x:v>
+        <x:v>Pontypridd</x:v>
       </x:c>
       <x:c r="B48" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str"/>
       <x:c r="D48" s="6" t="n">
-        <x:v>1850</x:v>
+        <x:v>1877</x:v>
       </x:c>
       <x:c r="E48" s="6" t="n">
-        <x:v>1887</x:v>
+        <x:v>1895</x:v>
       </x:c>
       <x:c r="F48" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G48" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="I48" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Research note only</x:v>
       </x:c>
       <x:c r="J48" s="5" t="str">
-        <x:v>CD 20; LR 12451 7</x:v>
+        <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K48" s="5" t="str"/>
       <x:c r="L48" s="5" t="str"/>
@@ -2165,89 +2175,89 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="4" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Rhymney</x:v>
       </x:c>
       <x:c r="B49" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str"/>
       <x:c r="D49" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1850</x:v>
       </x:c>
       <x:c r="E49" s="6" t="n">
         <x:v>1887</x:v>
       </x:c>
       <x:c r="F49" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G49" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="H49" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I49" s="5" t="str">
-        <x:v>Verified direct-FHC microfilm fallback source</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J49" s="5" t="str">
-        <x:v>Direct-FHC microfilm capture; photographed library identifier 1602; 57 authoritative images; source dates 1851-1887</x:v>
+        <x:v>CD 20; LR 12451 7</x:v>
       </x:c>
       <x:c r="K49" s="5" t="str"/>
       <x:c r="L49" s="5" t="str"/>
-      <x:c r="M49" s="5" t="str"/>
-      <x:c r="N49" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
+      <x:c r="M49" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N49" s="5" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="4" t="str">
-        <x:v>Stepaside</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="B50" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str"/>
       <x:c r="D50" s="6" t="n">
-        <x:v>1848</x:v>
+        <x:v>1851</x:v>
       </x:c>
       <x:c r="E50" s="6" t="n">
-        <x:v>1860</x:v>
+        <x:v>1887</x:v>
       </x:c>
       <x:c r="F50" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G50" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="H50" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="I50" s="5" t="str">
-        <x:v>Local CD only / verify with FamilySearch</x:v>
+        <x:v>Verified direct-FHC microfilm fallback source</x:v>
       </x:c>
       <x:c r="J50" s="5" t="str">
-        <x:v>CD 44; LR 12727 11; membership records 1848-1857; historical record and general minutes 1858-1860</x:v>
+        <x:v>Direct-FHC microfilm capture; photographed library identifier 1602; 57 authoritative images; source dates 1851-1887</x:v>
       </x:c>
       <x:c r="K50" s="5" t="str"/>
       <x:c r="L50" s="5" t="str"/>
-      <x:c r="M50" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
-      <x:c r="N50" s="5" t="str"/>
+      <x:c r="M50" s="5" t="str"/>
+      <x:c r="N50" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="4" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Stepaside</x:v>
       </x:c>
       <x:c r="B51" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str"/>
       <x:c r="D51" s="6" t="n">
-        <x:v>1853</x:v>
+        <x:v>1848</x:v>
       </x:c>
       <x:c r="E51" s="6" t="n">
-        <x:v>1859</x:v>
+        <x:v>1860</x:v>
       </x:c>
       <x:c r="F51" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2256,98 +2266,98 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="H51" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I51" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>Local CD only / verify with FamilySearch</x:v>
       </x:c>
       <x:c r="J51" s="5" t="str">
-        <x:v>CD 56; LR 12770 11; membership register 1853-1859; historical record and branch minutes 1853-1855; Film 104171 item 6</x:v>
+        <x:v>CD 44; LR 12727 11; membership records 1848-1857; historical record and general minutes 1858-1860</x:v>
       </x:c>
       <x:c r="K51" s="5" t="str"/>
       <x:c r="L51" s="5" t="str"/>
-      <x:c r="M51" s="5" t="str"/>
-      <x:c r="N51" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
-      </x:c>
+      <x:c r="M51" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N51" s="5" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="4" t="str">
-        <x:v>Swansea</x:v>
+        <x:v>Sutton Mountain</x:v>
       </x:c>
       <x:c r="B52" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C52" s="5" t="str">
-        <x:v>Abertawe; Abertawe (see Swansea)</x:v>
-      </x:c>
+      <x:c r="C52" s="5" t="str"/>
       <x:c r="D52" s="6" t="n">
-        <x:v>1852</x:v>
+        <x:v>1853</x:v>
       </x:c>
       <x:c r="E52" s="6" t="n">
-        <x:v>1879</x:v>
+        <x:v>1859</x:v>
       </x:c>
       <x:c r="F52" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G52" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H52" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="I52" s="5" t="str">
-        <x:v>Verified local source identity and collections</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J52" s="5" t="str">
-        <x:v>CD 32; LR 8863 7; CD 61; general minutes; Swansea / Abertawe source identity; Swansea Branch LR 8863 10; Wales2Utah research note</x:v>
+        <x:v>CD 56; LR 12770 11; membership register 1853-1859; historical record and branch minutes 1853-1855; Film 104171 item 6</x:v>
       </x:c>
       <x:c r="K52" s="5" t="str"/>
-      <x:c r="L52" s="5" t="str">
-        <x:v>Abertawe is the Welsh/historical source name for Swansea; the recovered LR 8863 10 description states that the branch was known as Abertawe until 1866.</x:v>
-      </x:c>
+      <x:c r="L52" s="5" t="str"/>
       <x:c r="M52" s="5" t="str"/>
-      <x:c r="N52" s="5" t="str"/>
+      <x:c r="N52" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="4" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="B53" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C53" s="5" t="str"/>
+      <x:c r="C53" s="5" t="str">
+        <x:v>Abertawe; Abertawe (see Swansea)</x:v>
+      </x:c>
       <x:c r="D53" s="6" t="n">
-        <x:v>1844</x:v>
+        <x:v>1852</x:v>
       </x:c>
       <x:c r="E53" s="6" t="n">
-        <x:v>1880</x:v>
+        <x:v>1879</x:v>
       </x:c>
       <x:c r="F53" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G53" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H53" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I53" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>Verified local source identity and collections</x:v>
       </x:c>
       <x:c r="J53" s="5" t="str">
-        <x:v>CD 16; LR 228 7; Film 104172 Item 1</x:v>
+        <x:v>CD 32; LR 8863 7; CD 61; general minutes; Swansea / Abertawe source identity; Swansea Branch LR 8863 10; Wales2Utah research note</x:v>
       </x:c>
       <x:c r="K53" s="5" t="str"/>
-      <x:c r="L53" s="5" t="str"/>
+      <x:c r="L53" s="5" t="str">
+        <x:v>Abertawe is the Welsh/historical source name for Swansea; the recovered LR 8863 10 description states that the branch was known as Abertawe until 1866.</x:v>
+      </x:c>
       <x:c r="M53" s="5" t="str"/>
-      <x:c r="N53" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
+      <x:c r="N53" s="5" t="str"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="4" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Treboeth</x:v>
       </x:c>
       <x:c r="B54" s="4" t="str">
         <x:v>Branch</x:v>
@@ -2357,7 +2367,7 @@
         <x:v>1844</x:v>
       </x:c>
       <x:c r="E54" s="6" t="n">
-        <x:v>1883</x:v>
+        <x:v>1880</x:v>
       </x:c>
       <x:c r="F54" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2372,7 +2382,7 @@
         <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J54" s="5" t="str">
-        <x:v>CD 5; LR 164 7; Film 104172 Items 2-3</x:v>
+        <x:v>CD 16; LR 228 7; Film 104172 Item 1</x:v>
       </x:c>
       <x:c r="K54" s="5" t="str"/>
       <x:c r="L54" s="5" t="str"/>
@@ -2383,17 +2393,17 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="4" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Tredegar</x:v>
       </x:c>
       <x:c r="B55" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str"/>
       <x:c r="D55" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1844</x:v>
       </x:c>
       <x:c r="E55" s="6" t="n">
-        <x:v>1873</x:v>
+        <x:v>1883</x:v>
       </x:c>
       <x:c r="F55" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2408,7 +2418,7 @@
         <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J55" s="5" t="str">
-        <x:v>CD 30; LR 12886 7; Film 104172 Item 4</x:v>
+        <x:v>CD 5; LR 164 7; Film 104172 Items 2-3</x:v>
       </x:c>
       <x:c r="K55" s="5" t="str"/>
       <x:c r="L55" s="5" t="str"/>
@@ -2419,19 +2429,17 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="4" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Treforest</x:v>
       </x:c>
       <x:c r="B56" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C56" s="5" t="str">
-        <x:v>Treorky</x:v>
-      </x:c>
+      <x:c r="C56" s="5" t="str"/>
       <x:c r="D56" s="6" t="n">
-        <x:v>1874</x:v>
+        <x:v>1851</x:v>
       </x:c>
       <x:c r="E56" s="6" t="n">
-        <x:v>1882</x:v>
+        <x:v>1873</x:v>
       </x:c>
       <x:c r="F56" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2443,34 +2451,36 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I56" s="5" t="str">
-        <x:v>Verified compound local source section</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J56" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound logical sections; 68 authoritative full-resolution images; Treorky minutes 1874 and membership register 1875-1882</x:v>
+        <x:v>CD 30; LR 12886 7; Film 104172 Item 4</x:v>
       </x:c>
       <x:c r="K56" s="5" t="str"/>
       <x:c r="L56" s="5" t="str"/>
       <x:c r="M56" s="5" t="str"/>
       <x:c r="N56" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168; https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="4" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="B57" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="C57" s="5" t="str"/>
+      <x:c r="C57" s="5" t="str">
+        <x:v>Treorky</x:v>
+      </x:c>
       <x:c r="D57" s="6" t="n">
-        <x:v>1849</x:v>
+        <x:v>1874</x:v>
       </x:c>
       <x:c r="E57" s="6" t="n">
-        <x:v>1853</x:v>
+        <x:v>1882</x:v>
       </x:c>
       <x:c r="F57" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G57" s="4" t="str">
         <x:v>No</x:v>
@@ -2479,36 +2489,34 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I57" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Verified compound local source section</x:v>
       </x:c>
       <x:c r="J57" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
+        <x:v>CD 34; LR 172 7 compound logical sections; 68 authoritative full-resolution images; Treorky minutes 1874 and membership register 1875-1882</x:v>
       </x:c>
       <x:c r="K57" s="5" t="str"/>
       <x:c r="L57" s="5" t="str"/>
-      <x:c r="M57" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M57" s="5" t="str"/>
       <x:c r="N57" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168; https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="4" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="B58" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str"/>
       <x:c r="D58" s="6" t="n">
-        <x:v>1847</x:v>
+        <x:v>1849</x:v>
       </x:c>
       <x:c r="E58" s="6" t="n">
-        <x:v>1901</x:v>
+        <x:v>1853</x:v>
       </x:c>
       <x:c r="F58" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="G58" s="4" t="str">
         <x:v>No</x:v>
@@ -2517,34 +2525,36 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I58" s="5" t="str">
-        <x:v>Matched: FamilySearch and local CD</x:v>
+        <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J58" s="5" t="str">
-        <x:v>CD 33; LR 165 7; Film 104172 Items 9-10</x:v>
+        <x:v>Photographed library identifier 859; compound PDF pages 4-5; Film 104172 Item 6</x:v>
       </x:c>
       <x:c r="K58" s="5" t="str"/>
       <x:c r="L58" s="5" t="str"/>
-      <x:c r="M58" s="5" t="str"/>
+      <x:c r="M58" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
       <x:c r="N58" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="4" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Twyn-yr-Odyn</x:v>
       </x:c>
       <x:c r="B59" s="4" t="str">
         <x:v>Branch</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str"/>
       <x:c r="D59" s="6" t="n">
-        <x:v>1851</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="E59" s="6" t="n">
-        <x:v>1883</x:v>
+        <x:v>1901</x:v>
       </x:c>
       <x:c r="F59" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G59" s="4" t="str">
         <x:v>No</x:v>
@@ -2553,39 +2563,39 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I59" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Matched: FamilySearch and local CD</x:v>
       </x:c>
       <x:c r="J59" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>CD 33; LR 165 7; Film 104172 Items 9-10</x:v>
       </x:c>
       <x:c r="K59" s="5" t="str"/>
       <x:c r="L59" s="5" t="str"/>
-      <x:c r="M59" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M59" s="5" t="str"/>
       <x:c r="N59" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="4" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Twyncarno</x:v>
       </x:c>
       <x:c r="B60" s="4" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="C60" s="5" t="str"/>
+        <x:v>Branch</x:v>
+      </x:c>
+      <x:c r="C60" s="5" t="str">
+        <x:v>Twyn Carno</x:v>
+      </x:c>
       <x:c r="D60" s="6" t="n">
-        <x:v>1850</x:v>
+        <x:v>1856</x:v>
       </x:c>
       <x:c r="E60" s="6" t="n">
-        <x:v>1922</x:v>
+        <x:v>1857</x:v>
       </x:c>
       <x:c r="F60" s="4" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G60" s="4" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H60" s="4" t="str">
         <x:v>Yes</x:v>
@@ -2594,7 +2604,7 @@
         <x:v>FamilySearch only / locate local record</x:v>
       </x:c>
       <x:c r="J60" s="5" t="str">
-        <x:v>Wales2Utah research note; Film 104172 Item 11</x:v>
+        <x:v>Captures 314-338; photographed library identifier 1602; 25 retained source frames; Film 104172 Items 7-8</x:v>
       </x:c>
       <x:c r="K60" s="5" t="str"/>
       <x:c r="L60" s="5" t="str"/>
@@ -2607,51 +2617,87 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="4" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Welsh Conference</x:v>
       </x:c>
       <x:c r="B61" s="4" t="str">
-        <x:v>Branch</x:v>
+        <x:v>Conference</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str"/>
       <x:c r="D61" s="6" t="n">
-        <x:v>1885</x:v>
+        <x:v>1850</x:v>
       </x:c>
       <x:c r="E61" s="6" t="n">
-        <x:v>1911</x:v>
+        <x:v>1922</x:v>
       </x:c>
       <x:c r="F61" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G61" s="4" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H61" s="4" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I61" s="5" t="str">
-        <x:v>FamilySearch only / locate local record</x:v>
+        <x:v>Verified local direct-FHC conference sources; Library 3118 incomplete</x:v>
       </x:c>
       <x:c r="J61" s="5" t="str">
-        <x:v>Film 104172 Item 12</x:v>
+        <x:v>Film 104172 item 11 context; Library 1614 early-1892; Library 3114 1887-1901; Library 3118 early-1911 partial capture; LR1001123 incomplete minutes, 1884; Wales2Utah research note; Film 104172 Item 11</x:v>
       </x:c>
       <x:c r="K61" s="5" t="str"/>
       <x:c r="L61" s="5" t="str"/>
-      <x:c r="M61" s="5" t="str">
-        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
-      </x:c>
+      <x:c r="M61" s="5" t="str"/>
       <x:c r="N61" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
       </x:c>
     </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="4" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="B62" s="4" t="str">
+        <x:v>Branch</x:v>
+      </x:c>
+      <x:c r="C62" s="5" t="str"/>
+      <x:c r="D62" s="6" t="n">
+        <x:v>1885</x:v>
+      </x:c>
+      <x:c r="E62" s="6" t="n">
+        <x:v>1911</x:v>
+      </x:c>
+      <x:c r="F62" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G62" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H62" s="4" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I62" s="5" t="str">
+        <x:v>FamilySearch only / locate local record</x:v>
+      </x:c>
+      <x:c r="J62" s="5" t="str">
+        <x:v>Film 104172 Item 12</x:v>
+      </x:c>
+      <x:c r="K62" s="5" t="str"/>
+      <x:c r="L62" s="5" t="str"/>
+      <x:c r="M62" s="5" t="str">
+        <x:v>Needs human review; absence from one source is not proof the branch or record was absent.</x:v>
+      </x:c>
+      <x:c r="N62" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="I2:I61">
+  <x:conditionalFormatting sqref="I2:I62">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="FamilySearch only"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Local CD only"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Matched"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78a506140f1a468c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea6b240e77d47bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3507,21 +3553,21 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="5" t="str">
-        <x:v>Abertillery</x:v>
+        <x:v>Cwmtillery</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>Abertillery</x:v>
+        <x:v>Cwmtillery</x:v>
       </x:c>
       <x:c r="C37" s="5" t="str"/>
       <x:c r="D37" s="5" t="str"/>
       <x:c r="E37" s="5" t="str">
-        <x:v>Recovered full-resolution compound source</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F37" s="5" t="str">
-        <x:v>1861-1866</x:v>
+        <x:v>1847-1857</x:v>
       </x:c>
       <x:c r="G37" s="5" t="str">
-        <x:v>CD 19; LR 195 7 compound section; images 00046-00057; 12 authoritative images</x:v>
+        <x:v>CD 8; LR 188 7; photographed library identifier 859; 69 authoritative full-resolution images</x:v>
       </x:c>
       <x:c r="H37" s="5" t="str"/>
       <x:c r="I37" s="5" t="str">
@@ -3530,21 +3576,21 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Trinant</x:v>
       </x:c>
       <x:c r="C38" s="5" t="str"/>
       <x:c r="D38" s="5" t="str"/>
       <x:c r="E38" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Direct-FHC microfilm recovery</x:v>
       </x:c>
       <x:c r="F38" s="5" t="str">
-        <x:v>1849-1876</x:v>
+        <x:v>1849-1853</x:v>
       </x:c>
       <x:c r="G38" s="5" t="str">
-        <x:v>CD 6; LR 198 7; 83 authoritative historical images</x:v>
+        <x:v>Photographed library identifier 859; compound PDF pages 4-5</x:v>
       </x:c>
       <x:c r="H38" s="5" t="str"/>
       <x:c r="I38" s="5" t="str">
@@ -3553,21 +3599,21 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="C39" s="5" t="str"/>
       <x:c r="D39" s="5" t="str"/>
       <x:c r="E39" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Direct-FHC microfilm recovery</x:v>
       </x:c>
       <x:c r="F39" s="5" t="str">
-        <x:v>1848-1878</x:v>
+        <x:v>1857-1862</x:v>
       </x:c>
       <x:c r="G39" s="5" t="str">
-        <x:v>CD 1; LR 182 7; source image/catalog prefix 1555; 66 authoritative images</x:v>
+        <x:v>Photographed library identifier 859; four bounded register frames within a nine-frame compound packet</x:v>
       </x:c>
       <x:c r="H39" s="5" t="str"/>
       <x:c r="I39" s="5" t="str">
@@ -3576,21 +3622,21 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="5" t="str">
-        <x:v>Brynmawr</x:v>
+        <x:v>Machen</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
-        <x:v>Brynmawr</x:v>
+        <x:v>Machen</x:v>
       </x:c>
       <x:c r="C40" s="5" t="str"/>
       <x:c r="D40" s="5" t="str"/>
       <x:c r="E40" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Direct-FHC microfilm recovery</x:v>
       </x:c>
       <x:c r="F40" s="5" t="str">
-        <x:v>1848-1868</x:v>
+        <x:v>1854-1865</x:v>
       </x:c>
       <x:c r="G40" s="5" t="str">
-        <x:v>CD 10; LR 215 7; 93 authoritative images</x:v>
+        <x:v>18 recovered PDF frames; photographed identifier unresolved as 1565 versus 1765</x:v>
       </x:c>
       <x:c r="H40" s="5" t="str"/>
       <x:c r="I40" s="5" t="str">
@@ -3599,21 +3645,21 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="5" t="str">
-        <x:v>Bryn</x:v>
+        <x:v>Twyn Carno</x:v>
       </x:c>
       <x:c r="B41" s="5" t="str">
-        <x:v>Bryntroedgam</x:v>
+        <x:v>Twyncarno</x:v>
       </x:c>
       <x:c r="C41" s="5" t="str"/>
       <x:c r="D41" s="5" t="str"/>
       <x:c r="E41" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Direct-FHC microfilm recovery</x:v>
       </x:c>
       <x:c r="F41" s="5" t="str">
-        <x:v>1847-1860</x:v>
+        <x:v>1856-1857</x:v>
       </x:c>
       <x:c r="G41" s="5" t="str">
-        <x:v>CD 13; LR 129 7; 44 authoritative images; source heading Bryn Branch / Canghen y Bryn</x:v>
+        <x:v>Captures 314-338; photographed library identifier 1602; 25 retained source frames</x:v>
       </x:c>
       <x:c r="H41" s="5" t="str"/>
       <x:c r="I41" s="5" t="str">
@@ -3622,21 +3668,21 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="5" t="str">
-        <x:v>Ebbro Vale</x:v>
+        <x:v>Welsh Conference</x:v>
       </x:c>
       <x:c r="B42" s="5" t="str">
-        <x:v>Ebbw Vale</x:v>
+        <x:v>Welsh Conference</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str"/>
       <x:c r="D42" s="5" t="str"/>
       <x:c r="E42" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Recovered direct-FHC microfilm components</x:v>
       </x:c>
       <x:c r="F42" s="5" t="str">
-        <x:v>1847-1864</x:v>
+        <x:v>1850-1922</x:v>
       </x:c>
       <x:c r="G42" s="5" t="str">
-        <x:v>CD 26; LR 9846 7; 76 authoritative images; historical/source spelling for Ebbw Vale</x:v>
+        <x:v>Film 104172 item 11 context; Library 1614 early-1892; Library 3114 1887-1901; Library 3118 early-1911 partial capture; LR1001123 incomplete minutes, 1884</x:v>
       </x:c>
       <x:c r="H42" s="5" t="str"/>
       <x:c r="I42" s="5" t="str">
@@ -3645,56 +3691,52 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="5" t="str">
-        <x:v>Gwaen Helygen</x:v>
+        <x:v>Cwmcillyn</x:v>
       </x:c>
       <x:c r="B43" s="5" t="str">
-        <x:v>Brynmawr</x:v>
+        <x:v>Cwmcillyn</x:v>
       </x:c>
       <x:c r="C43" s="5" t="str"/>
       <x:c r="D43" s="5" t="str"/>
       <x:c r="E43" s="5" t="str">
-        <x:v>Original CD contents description</x:v>
+        <x:v>2026 bounded local recovery audit</x:v>
       </x:c>
       <x:c r="F43" s="5" t="str">
-        <x:v>1848-1868</x:v>
+        <x:v>1847-1856</x:v>
       </x:c>
       <x:c r="G43" s="5" t="str">
-        <x:v>Historical/source name for Brynmawr</x:v>
+        <x:v>Film 104168 Item 12; no matching local image or PDF packet located</x:v>
       </x:c>
       <x:c r="H43" s="5" t="str"/>
-      <x:c r="I43" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+      <x:c r="I43" s="5" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="5" t="str">
-        <x:v>Cog</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="B44" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="C44" s="5" t="str"/>
       <x:c r="D44" s="5" t="str"/>
       <x:c r="E44" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>2026 bounded local recovery audit</x:v>
       </x:c>
       <x:c r="F44" s="5" t="str">
-        <x:v>1848-1876</x:v>
+        <x:v>1851-1886</x:v>
       </x:c>
       <x:c r="G44" s="5" t="str">
-        <x:v>CD 31; LR 109 7; 68 authoritative images; historical/source name for Cogan</x:v>
+        <x:v>DGS 106248102; indexing images 195-239; no matching local image or PDF packet located</x:v>
       </x:c>
       <x:c r="H44" s="5" t="str"/>
-      <x:c r="I44" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+      <x:c r="I44" s="5" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="5" t="str">
-        <x:v>Cefncoed-y-Cymar</x:v>
+        <x:v>Llansawel (Carmarthenshire)</x:v>
       </x:c>
       <x:c r="B45" s="5" t="str">
-        <x:v>Cefn Coed-y-Cymmer</x:v>
+        <x:v>Llansawel (Carmarthenshire)</x:v>
       </x:c>
       <x:c r="C45" s="5" t="str"/>
       <x:c r="D45" s="5" t="str"/>
@@ -3702,10 +3744,10 @@
         <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F45" s="5" t="str">
-        <x:v>1847-1864</x:v>
+        <x:v>1849-1855</x:v>
       </x:c>
       <x:c r="G45" s="5" t="str">
-        <x:v>CD 12; LR 176 7; 109 authoritative images; historical/source spelling for Cefn Coed-y-Cymmer</x:v>
+        <x:v>CD 14; LR 221 7; photographed library identifier 318; 28 authoritative images</x:v>
       </x:c>
       <x:c r="H45" s="5" t="str"/>
       <x:c r="I45" s="5" t="str">
@@ -3714,21 +3756,21 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="5" t="str">
-        <x:v>Altwen</x:v>
+        <x:v>Llansawel (Glamorgan)</x:v>
       </x:c>
       <x:c r="B46" s="5" t="str">
-        <x:v>Alltwen</x:v>
+        <x:v>Llansawel (Glamorgan)</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str"/>
       <x:c r="D46" s="5" t="str"/>
       <x:c r="E46" s="5" t="str">
-        <x:v>Local LR2257 membership register</x:v>
+        <x:v>Recovered full-resolution compound source section</x:v>
       </x:c>
       <x:c r="F46" s="5" t="str">
-        <x:v>1849-1859</x:v>
+        <x:v>1850-1889</x:v>
       </x:c>
       <x:c r="G46" s="5" t="str">
-        <x:v>LR 225 7; historical/source spelling of Alltwen</x:v>
+        <x:v>CD 18; LR 11759 7; explicit images 00009-00048; 40 authoritative in-place images</x:v>
       </x:c>
       <x:c r="H46" s="5" t="str"/>
       <x:c r="I46" s="5" t="str">
@@ -3737,21 +3779,21 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="5" t="str">
-        <x:v>Briton Ferry</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="B47" s="5" t="str">
-        <x:v>Britonferry</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str"/>
       <x:c r="D47" s="5" t="str"/>
       <x:c r="E47" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Direct-FHC microfilm recovery</x:v>
       </x:c>
       <x:c r="F47" s="5" t="str">
-        <x:v>1850-1853</x:v>
+        <x:v>Early to 1947</x:v>
       </x:c>
       <x:c r="G47" s="5" t="str">
-        <x:v>LR 11759 7; explicit Briton Ferry section, pages 43-46, in compound Llansawel/Swansea/Briton Ferry volume</x:v>
+        <x:v>10-page source packet; photographed library identifier 27560</x:v>
       </x:c>
       <x:c r="H47" s="5" t="str"/>
       <x:c r="I47" s="5" t="str">
@@ -3760,19 +3802,21 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="5" t="str">
-        <x:v>Pen-y-Darran</x:v>
+        <x:v>Abertillery</x:v>
       </x:c>
       <x:c r="B48" s="5" t="str">
-        <x:v>Pen-y-Darran</x:v>
+        <x:v>Abertillery</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str"/>
       <x:c r="D48" s="5" t="str"/>
       <x:c r="E48" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
-      </x:c>
-      <x:c r="F48" s="5" t="str"/>
+        <x:v>Recovered full-resolution compound source</x:v>
+      </x:c>
+      <x:c r="F48" s="5" t="str">
+        <x:v>1861-1866</x:v>
+      </x:c>
       <x:c r="G48" s="5" t="str">
-        <x:v>CD 36; two-page baptism list</x:v>
+        <x:v>CD 19; LR 195 7 compound section; images 00046-00057; 12 authoritative images</x:v>
       </x:c>
       <x:c r="H48" s="5" t="str"/>
       <x:c r="I48" s="5" t="str">
@@ -3781,21 +3825,21 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="5" t="str">
-        <x:v>Gymmer</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="B49" s="5" t="str">
-        <x:v>Cymmer</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str"/>
       <x:c r="D49" s="5" t="str"/>
       <x:c r="E49" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F49" s="5" t="str">
-        <x:v>1852-1857; 1863</x:v>
+        <x:v>1849-1876</x:v>
       </x:c>
       <x:c r="G49" s="5" t="str">
-        <x:v>CD 59; meeting transcription checklist</x:v>
+        <x:v>CD 6; LR 198 7; 83 authoritative historical images</x:v>
       </x:c>
       <x:c r="H49" s="5" t="str"/>
       <x:c r="I49" s="5" t="str">
@@ -3804,21 +3848,21 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="5" t="str">
-        <x:v>Stepaside</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="B50" s="5" t="str">
-        <x:v>Stepaside</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str"/>
       <x:c r="D50" s="5" t="str"/>
       <x:c r="E50" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F50" s="5" t="str">
-        <x:v>1848-1860</x:v>
+        <x:v>1848-1878</x:v>
       </x:c>
       <x:c r="G50" s="5" t="str">
-        <x:v>CD 44; LR 12727 11; membership records 1848-1857; historical record and general minutes 1858-1860</x:v>
+        <x:v>CD 1; LR 182 7; source image/catalog prefix 1555; 66 authoritative images</x:v>
       </x:c>
       <x:c r="H50" s="5" t="str"/>
       <x:c r="I50" s="5" t="str">
@@ -3827,21 +3871,21 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Brynmawr</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Brynmawr</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str"/>
       <x:c r="D51" s="5" t="str"/>
       <x:c r="E51" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F51" s="5" t="str">
-        <x:v>1853-1859</x:v>
+        <x:v>1848-1868</x:v>
       </x:c>
       <x:c r="G51" s="5" t="str">
-        <x:v>CD 56; LR 12770 11; membership register 1853-1859; historical record and branch minutes 1853-1855</x:v>
+        <x:v>CD 10; LR 215 7; 93 authoritative images</x:v>
       </x:c>
       <x:c r="H51" s="5" t="str"/>
       <x:c r="I51" s="5" t="str">
@@ -3850,21 +3894,21 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="5" t="str">
-        <x:v>Swansea</x:v>
+        <x:v>Bryn</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>Swansea</x:v>
+        <x:v>Bryntroedgam</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str"/>
       <x:c r="D52" s="5" t="str"/>
       <x:c r="E52" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F52" s="5" t="str">
-        <x:v>1852-1854</x:v>
+        <x:v>1847-1860</x:v>
       </x:c>
       <x:c r="G52" s="5" t="str">
-        <x:v>CD 61; general minutes</x:v>
+        <x:v>CD 13; LR 129 7; 44 authoritative images; source heading Bryn Branch / Canghen y Bryn</x:v>
       </x:c>
       <x:c r="H52" s="5" t="str"/>
       <x:c r="I52" s="5" t="str">
@@ -3873,21 +3917,21 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="5" t="str">
-        <x:v>Pontypool</x:v>
+        <x:v>Ebbro Vale</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>Pontypool</x:v>
+        <x:v>Ebbw Vale</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str"/>
       <x:c r="D53" s="5" t="str"/>
       <x:c r="E53" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F53" s="5" t="str">
-        <x:v>1857-1884</x:v>
+        <x:v>1847-1864</x:v>
       </x:c>
       <x:c r="G53" s="5" t="str">
-        <x:v>CD 62; general minutes</x:v>
+        <x:v>CD 26; LR 9846 7; 76 authoritative images; historical/source spelling for Ebbw Vale</x:v>
       </x:c>
       <x:c r="H53" s="5" t="str"/>
       <x:c r="I53" s="5" t="str">
@@ -3896,21 +3940,21 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="5" t="str">
-        <x:v>Abersychan</x:v>
+        <x:v>Gwaen Helygen</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>Abersychan</x:v>
+        <x:v>Brynmawr</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str"/>
       <x:c r="D54" s="5" t="str"/>
       <x:c r="E54" s="5" t="str">
-        <x:v>2007 meeting transcription checklist</x:v>
+        <x:v>Original CD contents description</x:v>
       </x:c>
       <x:c r="F54" s="5" t="str">
-        <x:v>1889</x:v>
+        <x:v>1848-1868</x:v>
       </x:c>
       <x:c r="G54" s="5" t="str">
-        <x:v>CD 62; general minutes</x:v>
+        <x:v>Historical/source name for Brynmawr</x:v>
       </x:c>
       <x:c r="H54" s="5" t="str"/>
       <x:c r="I54" s="5" t="str">
@@ -3919,40 +3963,44 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="5" t="str">
-        <x:v>Festiniog</x:v>
+        <x:v>Cog</x:v>
       </x:c>
       <x:c r="B55" s="5" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str"/>
       <x:c r="D55" s="5" t="str"/>
       <x:c r="E55" s="5" t="str">
-        <x:v>Local membership record images</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F55" s="5" t="str">
-        <x:v>1848-1856</x:v>
+        <x:v>1848-1876</x:v>
       </x:c>
       <x:c r="G55" s="5" t="str">
-        <x:v>Ffestiniog membership record book integrated into local archive; surviving title uses Festiniog; 94 unique viewer images</x:v>
+        <x:v>CD 31; LR 109 7; 68 authoritative images; historical/source name for Cogan</x:v>
       </x:c>
       <x:c r="H55" s="5" t="str"/>
-      <x:c r="I55" s="5" t="str"/>
+      <x:c r="I55" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="5" t="str">
-        <x:v>Abertawe</x:v>
+        <x:v>Cefncoed-y-Cymar</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>Swansea</x:v>
+        <x:v>Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str"/>
       <x:c r="D56" s="5" t="str"/>
       <x:c r="E56" s="5" t="str">
-        <x:v>Recovered Swansea source description and Welsh source heading</x:v>
-      </x:c>
-      <x:c r="F56" s="5" t="str"/>
+        <x:v>Recovered full-resolution local source</x:v>
+      </x:c>
+      <x:c r="F56" s="5" t="str">
+        <x:v>1847-1864</x:v>
+      </x:c>
       <x:c r="G56" s="5" t="str">
-        <x:v>Swansea / Abertawe source identity; Swansea Branch LR 8863 10</x:v>
+        <x:v>CD 12; LR 176 7; 109 authoritative images; historical/source spelling for Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="H56" s="5" t="str"/>
       <x:c r="I56" s="5" t="str">
@@ -3961,21 +4009,21 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="5" t="str">
-        <x:v>Coal Brook Vale</x:v>
+        <x:v>Altwen</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>Coalbrookvale</x:v>
+        <x:v>Alltwen</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str"/>
       <x:c r="D57" s="5" t="str"/>
       <x:c r="E57" s="5" t="str">
-        <x:v>Recovered full-resolution compound source</x:v>
+        <x:v>Local LR2257 membership register</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>1856-1867</x:v>
+        <x:v>1849-1859</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
-        <x:v>CD 24; LR 174 7 compound section; 83 authoritative images; membership registers 00080-00137</x:v>
+        <x:v>LR 225 7; historical/source spelling of Alltwen</x:v>
       </x:c>
       <x:c r="H57" s="5" t="str"/>
       <x:c r="I57" s="5" t="str">
@@ -3984,281 +4032,291 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str"/>
       <x:c r="D58" s="5" t="str"/>
       <x:c r="E58" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Welsh Saints Project historical resource</x:v>
       </x:c>
       <x:c r="F58" s="5" t="str">
-        <x:v>1847-1869</x:v>
+        <x:v>1840-1842</x:v>
       </x:c>
       <x:c r="G58" s="5" t="str">
-        <x:v>CD 15; project LR1687; historical/library identifier 871; 60 authoritative images</x:v>
-      </x:c>
-      <x:c r="H58" s="5" t="str"/>
-      <x:c r="I58" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+        <x:v>Overton: The First LDS Branch in Wales; organized 30 October 1840; earliest documented branch in Wales</x:v>
+      </x:c>
+      <x:c r="H58" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Resource_Info.aspx?id=24497</x:v>
+      </x:c>
+      <x:c r="I58" s="5" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Owrtyn</x:v>
       </x:c>
       <x:c r="B59" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str"/>
       <x:c r="D59" s="5" t="str"/>
       <x:c r="E59" s="5" t="str">
-        <x:v>Recovered full-resolution local sources</x:v>
+        <x:v>Welsh Saints Project place-name evidence</x:v>
       </x:c>
       <x:c r="F59" s="5" t="str">
-        <x:v>1847-1860</x:v>
+        <x:v>1840-1842</x:v>
       </x:c>
       <x:c r="G59" s="5" t="str">
-        <x:v>CD 23 / CR 11343 11 V.1; CD 58 / CR 11343 11 V.2; 272 authoritative historical images</x:v>
-      </x:c>
-      <x:c r="H59" s="5" t="str"/>
-      <x:c r="I59" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+        <x:v>Welsh spelling used in Welsh Saints person records for Overton, Flintshire</x:v>
+      </x:c>
+      <x:c r="H59" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Resource_Info.aspx?id=24497</x:v>
+      </x:c>
+      <x:c r="I59" s="5" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="B60" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Overton</x:v>
       </x:c>
       <x:c r="C60" s="5" t="str"/>
       <x:c r="D60" s="5" t="str"/>
       <x:c r="E60" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Ronald D. Dennis historical narrative</x:v>
       </x:c>
       <x:c r="F60" s="5" t="str">
-        <x:v>1849-1866</x:v>
+        <x:v>1840</x:v>
       </x:c>
       <x:c r="G60" s="5" t="str">
-        <x:v>CD 22; project LR 113 7; photographed library identifier 870; 45 authoritative full-resolution images</x:v>
+        <x:v>Opposition to the Gospel Message in Wales, PDF page 23; missionaries arrived 16 October and organized a branch 30 October 1840</x:v>
       </x:c>
       <x:c r="H60" s="5" t="str"/>
-      <x:c r="I60" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+      <x:c r="I60" s="5" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="5" t="str">
-        <x:v>Castell Nedd</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="B61" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str"/>
       <x:c r="D61" s="5" t="str"/>
       <x:c r="E61" s="5" t="str">
-        <x:v>Recovered full-resolution local source</x:v>
+        <x:v>Hugh and Mary Owens Roberts biographical history</x:v>
       </x:c>
       <x:c r="F61" s="5" t="str">
-        <x:v>1849-1884</x:v>
+        <x:v>1849-1864</x:v>
       </x:c>
       <x:c r="G61" s="5" t="str">
-        <x:v>CD 2; project LR 196 7; photographed source/library identifier 1544; 112 authoritative full-resolution images</x:v>
-      </x:c>
-      <x:c r="H61" s="5" t="str"/>
-      <x:c r="I61" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+        <x:v>Abel Evans organized a six-member branch; Hugh Roberts served as presiding elder and kept the branch record until emigrating in 1864</x:v>
+      </x:c>
+      <x:c r="H61" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Immigrant_View.aspx?id=806</x:v>
+      </x:c>
+      <x:c r="I61" s="5" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="5" t="str">
-        <x:v>Castellned</x:v>
+        <x:v>Eglwys Fach</x:v>
       </x:c>
       <x:c r="B62" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="C62" s="5" t="str"/>
       <x:c r="D62" s="5" t="str"/>
       <x:c r="E62" s="5" t="str">
-        <x:v>Historical source heading</x:v>
+        <x:v>Welsh Saints Project place-name evidence</x:v>
       </x:c>
       <x:c r="F62" s="5" t="str">
-        <x:v>1849-1883</x:v>
+        <x:v>1849-1864</x:v>
       </x:c>
       <x:c r="G62" s="5" t="str">
-        <x:v>CD 2; photographed source/library identifier 1544</x:v>
-      </x:c>
-      <x:c r="H62" s="5" t="str"/>
-      <x:c r="I62" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+        <x:v>Historical/source spelling used in Hugh Roberts family records</x:v>
+      </x:c>
+      <x:c r="H62" s="5" t="str">
+        <x:v>https://welshsaints.byu.edu/Immigrant_View.aspx?id=806</x:v>
+      </x:c>
+      <x:c r="I62" s="5" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Eglwys Bach</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="C63" s="5" t="str"/>
       <x:c r="D63" s="5" t="str"/>
       <x:c r="E63" s="5" t="str">
-        <x:v>Recovered direct-FHC microfilm source</x:v>
+        <x:v>Historical spacing variant</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
-        <x:v>1851-1887</x:v>
+        <x:v>1849-1864</x:v>
       </x:c>
       <x:c r="G63" s="5" t="str">
-        <x:v>Direct-FHC microfilm capture; library identifier 1602; 57 authoritative images</x:v>
+        <x:v>Variant spacing retained for discovery</x:v>
       </x:c>
       <x:c r="H63" s="5" t="str"/>
-      <x:c r="I63" s="5" t="str">
-        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
-      </x:c>
+      <x:c r="I63" s="5" t="str"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="5" t="str">
-        <x:v>Pendoylon</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
-        <x:v>Pendoylon</x:v>
+        <x:v>Eglwysbach</x:v>
       </x:c>
       <x:c r="C64" s="5" t="str"/>
       <x:c r="D64" s="5" t="str"/>
       <x:c r="E64" s="5" t="str">
-        <x:v>2022 Wales indexing-project branch map</x:v>
+        <x:v>Zion's Trumpet conference report</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
-        <x:v>1851-1886</x:v>
+        <x:v>1854</x:v>
       </x:c>
       <x:c r="G64" s="5" t="str">
-        <x:v>DGS 106248102; indexing images 195-239; WALES (Country), Part 5</x:v>
+        <x:v>Conwy Valley Conference held at Eglwysbach, 28 May 1854; five branches and 98 members reported for the conference</x:v>
       </x:c>
       <x:c r="H64" s="5" t="str"/>
-      <x:c r="I64" s="5" t="str"/>
+      <x:c r="I64" s="5" t="str">
+        <x:v>resources/books/Zions Trumpet (1854).pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="5" t="str">
-        <x:v>Pendoylan</x:v>
+        <x:v>Briton Ferry</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
-        <x:v>Pendoylon</x:v>
+        <x:v>Britonferry</x:v>
       </x:c>
       <x:c r="C65" s="5" t="str"/>
       <x:c r="D65" s="5" t="str"/>
       <x:c r="E65" s="5" t="str">
-        <x:v>Ron Dennis typed conference material</x:v>
-      </x:c>
-      <x:c r="F65" s="5" t="str"/>
+        <x:v>2007 meeting transcription checklist</x:v>
+      </x:c>
+      <x:c r="F65" s="5" t="str">
+        <x:v>1850-1853</x:v>
+      </x:c>
       <x:c r="G65" s="5" t="str">
-        <x:v>Historical/source spelling in typed Cardiff conference records</x:v>
+        <x:v>LR 11759 7; explicit Briton Ferry section, pages 43-46, in compound Llansawel/Swansea/Briton Ferry volume</x:v>
       </x:c>
       <x:c r="H65" s="5" t="str"/>
-      <x:c r="I65" s="5" t="str"/>
+      <x:c r="I65" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="5" t="str">
-        <x:v>Llanellyd</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Pen-y-Darran</x:v>
       </x:c>
       <x:c r="C66" s="5" t="str"/>
       <x:c r="D66" s="5" t="str"/>
       <x:c r="E66" s="5" t="str">
-        <x:v>Historical structural image</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str"/>
       <x:c r="G66" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound volume</x:v>
+        <x:v>CD 36; two-page baptism list</x:v>
       </x:c>
       <x:c r="H66" s="5" t="str"/>
-      <x:c r="I66" s="5" t="str"/>
+      <x:c r="I66" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Gymmer</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Cymmer</x:v>
       </x:c>
       <x:c r="C67" s="5" t="str"/>
       <x:c r="D67" s="5" t="str"/>
       <x:c r="E67" s="5" t="str">
-        <x:v>Recovered full-resolution compound source</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
-        <x:v>1850-1857</x:v>
+        <x:v>1852-1857; 1863</x:v>
       </x:c>
       <x:c r="G67" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound section; internal pages 1-5; 10 authoritative images</x:v>
+        <x:v>CD 59; meeting transcription checklist</x:v>
       </x:c>
       <x:c r="H67" s="5" t="str"/>
-      <x:c r="I67" s="5" t="str"/>
+      <x:c r="I67" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="5" t="str">
-        <x:v>Cwmsaerbren</x:v>
+        <x:v>Stepaside</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
-        <x:v>Cwm Saerbren</x:v>
+        <x:v>Stepaside</x:v>
       </x:c>
       <x:c r="C68" s="5" t="str"/>
       <x:c r="D68" s="5" t="str"/>
       <x:c r="E68" s="5" t="str">
-        <x:v>Historical structural image</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F68" s="5" t="str">
-        <x:v>1858-1874</x:v>
+        <x:v>1848-1860</x:v>
       </x:c>
       <x:c r="G68" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound section; 38 authoritative images; LR 11150 separate catalog reference not connected</x:v>
+        <x:v>CD 44; LR 12727 11; membership records 1848-1857; historical record and general minutes 1858-1860</x:v>
       </x:c>
       <x:c r="H68" s="5" t="str"/>
-      <x:c r="I68" s="5" t="str"/>
+      <x:c r="I68" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="5" t="str">
-        <x:v>Treorky</x:v>
+        <x:v>Sutton Mountain</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Sutton Mountain</x:v>
       </x:c>
       <x:c r="C69" s="5" t="str"/>
       <x:c r="D69" s="5" t="str"/>
       <x:c r="E69" s="5" t="str">
-        <x:v>Recovered full-resolution compound source</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
-        <x:v>1874-1882</x:v>
+        <x:v>1853-1859</x:v>
       </x:c>
       <x:c r="G69" s="5" t="str">
-        <x:v>CD 34; LR 172 7 compound sections; 68 virtual images</x:v>
+        <x:v>CD 56; LR 12770 11; membership register 1853-1859; historical record and branch minutes 1853-1855</x:v>
       </x:c>
       <x:c r="H69" s="5" t="str"/>
-      <x:c r="I69" s="5" t="str"/>
+      <x:c r="I69" s="5" t="str">
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="C70" s="5" t="str"/>
       <x:c r="D70" s="5" t="str"/>
       <x:c r="E70" s="5" t="str">
-        <x:v>Recovered CD 11 source labels</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F70" s="5" t="str">
-        <x:v>1847-1868</x:v>
+        <x:v>1852-1854</x:v>
       </x:c>
       <x:c r="G70" s="5" t="str">
-        <x:v>CD 11; source label 1577; recovered folder LR 11757 7; filename prefix LR 12451 7 (unresolved conflict)</x:v>
+        <x:v>CD 61; general minutes</x:v>
       </x:c>
       <x:c r="H70" s="5" t="str"/>
       <x:c r="I70" s="5" t="str">
@@ -4267,30 +4325,30 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="5" t="str">
-        <x:v>Abersycan (1887-1889)</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
-        <x:v>Abersychan</x:v>
+        <x:v>Pontypool</x:v>
       </x:c>
       <x:c r="C71" s="5" t="str"/>
       <x:c r="D71" s="5" t="str"/>
       <x:c r="E71" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F71" s="5" t="str">
-        <x:v>1887-1889</x:v>
+        <x:v>1857-1884</x:v>
       </x:c>
       <x:c r="G71" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="H71" s="5" t="str"/>
       <x:c r="I71" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersycan_(1887-1889).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="5" t="str">
-        <x:v>Abersychan (1848-1876)</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
         <x:v>Abersychan</x:v>
@@ -4298,434 +4356,426 @@
       <x:c r="C72" s="5" t="str"/>
       <x:c r="D72" s="5" t="str"/>
       <x:c r="E72" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>2007 meeting transcription checklist</x:v>
       </x:c>
       <x:c r="F72" s="5" t="str">
-        <x:v>1848-1876</x:v>
+        <x:v>1889</x:v>
       </x:c>
       <x:c r="G72" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 62; general minutes</x:v>
       </x:c>
       <x:c r="H72" s="5" t="str"/>
       <x:c r="I72" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersychan_(1848-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="5" t="str">
-        <x:v>Abertawe (see Swansea)</x:v>
+        <x:v>Festiniog</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
-        <x:v>Swansea</x:v>
-      </x:c>
-      <x:c r="C73" s="5" t="str">
-        <x:v>Swansea</x:v>
-      </x:c>
-      <x:c r="D73" s="5" t="str">
-        <x:v>See Swansea — possible rename, merger, transfer, or cross-reference; verify before classifying.</x:v>
-      </x:c>
+        <x:v>Ffestiniog</x:v>
+      </x:c>
+      <x:c r="C73" s="5" t="str"/>
+      <x:c r="D73" s="5" t="str"/>
       <x:c r="E73" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F73" s="5" t="str"/>
+        <x:v>Local membership record images</x:v>
+      </x:c>
+      <x:c r="F73" s="5" t="str">
+        <x:v>1848-1856</x:v>
+      </x:c>
       <x:c r="G73" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>Ffestiniog membership record book integrated into local archive; surviving title uses Festiniog; 94 unique viewer images</x:v>
       </x:c>
       <x:c r="H73" s="5" t="str"/>
-      <x:c r="I73" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertawe_(see_Swansea).htm</x:v>
-      </x:c>
+      <x:c r="I73" s="5" t="str"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="5" t="str">
-        <x:v>Abertillery (1861-1866)</x:v>
+        <x:v>Abertawe</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
-        <x:v>Abertillery</x:v>
+        <x:v>Swansea</x:v>
       </x:c>
       <x:c r="C74" s="5" t="str"/>
       <x:c r="D74" s="5" t="str"/>
       <x:c r="E74" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F74" s="5" t="str">
-        <x:v>1861-1866</x:v>
-      </x:c>
+        <x:v>Recovered Swansea source description and Welsh source heading</x:v>
+      </x:c>
+      <x:c r="F74" s="5" t="str"/>
       <x:c r="G74" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>Swansea / Abertawe source identity; Swansea Branch LR 8863 10</x:v>
       </x:c>
       <x:c r="H74" s="5" t="str"/>
       <x:c r="I74" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertillery_(1861-1866).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="5" t="str">
-        <x:v>Alltwen (1849-1859)</x:v>
+        <x:v>Coal Brook Vale</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
-        <x:v>Alltwen</x:v>
+        <x:v>Coalbrookvale</x:v>
       </x:c>
       <x:c r="C75" s="5" t="str"/>
       <x:c r="D75" s="5" t="str"/>
       <x:c r="E75" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution compound source</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
-        <x:v>1849-1859</x:v>
+        <x:v>1856-1867</x:v>
       </x:c>
       <x:c r="G75" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 24; LR 174 7 compound section; 83 authoritative images; membership registers 00080-00137</x:v>
       </x:c>
       <x:c r="H75" s="5" t="str"/>
       <x:c r="I75" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Alltwen_(1849-1859).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="5" t="str">
-        <x:v>Brechfa (1846-1868)</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
-        <x:v>Brechfa</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="C76" s="5" t="str"/>
       <x:c r="D76" s="5" t="str"/>
       <x:c r="E76" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F76" s="5" t="str">
-        <x:v>1846-1868</x:v>
+        <x:v>1847-1869</x:v>
       </x:c>
       <x:c r="G76" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 15; project LR1687; historical/library identifier 871; 60 authoritative images</x:v>
       </x:c>
       <x:c r="H76" s="5" t="str"/>
       <x:c r="I76" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Brechfa_(1846-1868).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="5" t="str">
-        <x:v>Cardiff (1849-1855)</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="C77" s="5" t="str"/>
       <x:c r="D77" s="5" t="str"/>
       <x:c r="E77" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution local sources</x:v>
       </x:c>
       <x:c r="F77" s="5" t="str">
-        <x:v>1849-1855</x:v>
+        <x:v>1847-1860</x:v>
       </x:c>
       <x:c r="G77" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 23 / CR 11343 11 V.1; CD 58 / CR 11343 11 V.2; 272 authoritative historical images</x:v>
       </x:c>
       <x:c r="H77" s="5" t="str"/>
       <x:c r="I77" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1849-1855).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="5" t="str">
-        <x:v>Cardiff (1854-1876)</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="C78" s="5" t="str"/>
       <x:c r="D78" s="5" t="str"/>
       <x:c r="E78" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F78" s="5" t="str">
-        <x:v>1854-1876</x:v>
+        <x:v>1849-1866</x:v>
       </x:c>
       <x:c r="G78" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 22; project LR 113 7; photographed library identifier 870; 45 authoritative full-resolution images</x:v>
       </x:c>
       <x:c r="H78" s="5" t="str"/>
       <x:c r="I78" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1854-1876).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="5" t="str">
-        <x:v>Cardiff (1931-1947)</x:v>
+        <x:v>Castell Nedd</x:v>
       </x:c>
       <x:c r="B79" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C79" s="5" t="str"/>
       <x:c r="D79" s="5" t="str"/>
       <x:c r="E79" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution local source</x:v>
       </x:c>
       <x:c r="F79" s="5" t="str">
-        <x:v>1931-1947</x:v>
+        <x:v>1849-1884</x:v>
       </x:c>
       <x:c r="G79" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 2; project LR 196 7; photographed source/library identifier 1544; 112 authoritative full-resolution images</x:v>
       </x:c>
       <x:c r="H79" s="5" t="str"/>
       <x:c r="I79" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1931-1947).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="5" t="str">
-        <x:v>Cardiff (Early to 1917, 1919)</x:v>
+        <x:v>Castellned</x:v>
       </x:c>
       <x:c r="B80" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C80" s="5" t="str"/>
       <x:c r="D80" s="5" t="str"/>
       <x:c r="E80" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Historical source heading</x:v>
       </x:c>
       <x:c r="F80" s="5" t="str">
-        <x:v>1917-1919</x:v>
+        <x:v>1849-1883</x:v>
       </x:c>
       <x:c r="G80" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 2; photographed source/library identifier 1544</x:v>
       </x:c>
       <x:c r="H80" s="5" t="str"/>
       <x:c r="I80" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(Early_to_1917,_1919).htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="5" t="str">
-        <x:v>Cardiff Branch</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="B81" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Rhymney English</x:v>
       </x:c>
       <x:c r="C81" s="5" t="str"/>
       <x:c r="D81" s="5" t="str"/>
       <x:c r="E81" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F81" s="5" t="str"/>
+        <x:v>Recovered direct-FHC microfilm source</x:v>
+      </x:c>
+      <x:c r="F81" s="5" t="str">
+        <x:v>1851-1887</x:v>
+      </x:c>
       <x:c r="G81" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>Direct-FHC microfilm capture; library identifier 1602; 57 authoritative images</x:v>
       </x:c>
       <x:c r="H81" s="5" t="str"/>
       <x:c r="I81" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_Branch.htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="B82" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="C82" s="5" t="str"/>
       <x:c r="D82" s="5" t="str"/>
       <x:c r="E82" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F82" s="5" t="str"/>
+        <x:v>2022 Wales indexing-project branch map</x:v>
+      </x:c>
+      <x:c r="F82" s="5" t="str">
+        <x:v>1851-1886</x:v>
+      </x:c>
       <x:c r="G82" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>DGS 106248102; indexing images 195-239; WALES (Country), Part 5</x:v>
       </x:c>
       <x:c r="H82" s="5" t="str"/>
-      <x:c r="I82" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Castell_Nedd_(Neath).htm</x:v>
-      </x:c>
+      <x:c r="I82" s="5" t="str"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="5" t="str">
-        <x:v>Cefncoed-y-Cymar (1847-1864)</x:v>
+        <x:v>Pendoylan</x:v>
       </x:c>
       <x:c r="B83" s="5" t="str">
-        <x:v>Cefn Coed-y-Cymmer</x:v>
+        <x:v>Pendoylon</x:v>
       </x:c>
       <x:c r="C83" s="5" t="str"/>
       <x:c r="D83" s="5" t="str"/>
       <x:c r="E83" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F83" s="5" t="str">
-        <x:v>1847-1864</x:v>
-      </x:c>
+        <x:v>Ron Dennis typed conference material</x:v>
+      </x:c>
+      <x:c r="F83" s="5" t="str"/>
       <x:c r="G83" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>Historical/source spelling in typed Cardiff conference records</x:v>
       </x:c>
       <x:c r="H83" s="5" t="str"/>
-      <x:c r="I83" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cefncoed-y-Cymar_(1847-1864).htm</x:v>
-      </x:c>
+      <x:c r="I83" s="5" t="str"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="5" t="str">
-        <x:v>Coal Brock Vale (1856-1867)</x:v>
+        <x:v>Llanellyd</x:v>
       </x:c>
       <x:c r="B84" s="5" t="str">
-        <x:v>Coalbrookvale</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="C84" s="5" t="str"/>
       <x:c r="D84" s="5" t="str"/>
       <x:c r="E84" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F84" s="5" t="str">
-        <x:v>1856-1867</x:v>
-      </x:c>
+        <x:v>Historical structural image</x:v>
+      </x:c>
+      <x:c r="F84" s="5" t="str"/>
       <x:c r="G84" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 34; LR 172 7 compound volume</x:v>
       </x:c>
       <x:c r="H84" s="5" t="str"/>
-      <x:c r="I84" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Coal_Brock_Vale_(1856-1867).htm</x:v>
-      </x:c>
+      <x:c r="I84" s="5" t="str"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="5" t="str">
-        <x:v>Cog (1848-1876)</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="B85" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="C85" s="5" t="str"/>
       <x:c r="D85" s="5" t="str"/>
       <x:c r="E85" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution compound source</x:v>
       </x:c>
       <x:c r="F85" s="5" t="str">
-        <x:v>1848-1876</x:v>
+        <x:v>1850-1857</x:v>
       </x:c>
       <x:c r="G85" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 34; LR 172 7 compound section; internal pages 1-5; 10 authoritative images</x:v>
       </x:c>
       <x:c r="H85" s="5" t="str"/>
-      <x:c r="I85" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cog_(1848-1876).htm</x:v>
-      </x:c>
+      <x:c r="I85" s="5" t="str"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="5" t="str">
-        <x:v>Crumlin (1857-1862)</x:v>
+        <x:v>Cwmsaerbren</x:v>
       </x:c>
       <x:c r="B86" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Cwm Saerbren</x:v>
       </x:c>
       <x:c r="C86" s="5" t="str"/>
       <x:c r="D86" s="5" t="str"/>
       <x:c r="E86" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Historical structural image</x:v>
       </x:c>
       <x:c r="F86" s="5" t="str">
-        <x:v>1857-1862</x:v>
+        <x:v>1858-1874</x:v>
       </x:c>
       <x:c r="G86" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 34; LR 172 7 compound section; 38 authoritative images; LR 11150 separate catalog reference not connected</x:v>
       </x:c>
       <x:c r="H86" s="5" t="str"/>
-      <x:c r="I86" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Crumlin_(1857-1862).htm</x:v>
-      </x:c>
+      <x:c r="I86" s="5" t="str"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="5" t="str">
-        <x:v>Cuffern Mountain (1849-1876)</x:v>
+        <x:v>Treorky</x:v>
       </x:c>
       <x:c r="B87" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Treorchy</x:v>
       </x:c>
       <x:c r="C87" s="5" t="str"/>
       <x:c r="D87" s="5" t="str"/>
       <x:c r="E87" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
+        <x:v>Recovered full-resolution compound source</x:v>
       </x:c>
       <x:c r="F87" s="5" t="str">
-        <x:v>1849-1876</x:v>
+        <x:v>1874-1882</x:v>
       </x:c>
       <x:c r="G87" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 34; LR 172 7 compound sections; 68 virtual images</x:v>
       </x:c>
       <x:c r="H87" s="5" t="str"/>
-      <x:c r="I87" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cuffern_Mountain_(1849-1876).htm</x:v>
-      </x:c>
+      <x:c r="I87" s="5" t="str"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="5" t="str">
-        <x:v>Cwm Celin</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="B88" s="5" t="str">
-        <x:v>Cwm Celyn</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C88" s="5" t="str"/>
       <x:c r="D88" s="5" t="str"/>
       <x:c r="E88" s="5" t="str">
-        <x:v>Recovered RoboHelp branch note</x:v>
-      </x:c>
-      <x:c r="F88" s="5" t="str"/>
+        <x:v>Recovered CD 11 source labels</x:v>
+      </x:c>
+      <x:c r="F88" s="5" t="str">
+        <x:v>1847-1868</x:v>
+      </x:c>
       <x:c r="G88" s="5" t="str">
-        <x:v>Wales2Utah research note</x:v>
+        <x:v>CD 11; source label 1577; recovered folder LR 11757 7; filename prefix LR 12451 7 (unresolved conflict)</x:v>
       </x:c>
       <x:c r="H88" s="5" t="str"/>
       <x:c r="I88" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwm_Celin.htm</x:v>
+        <x:v>C:\Users\kenro\Documents\Codex\LDSWelshMembers\resources\source-cds</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="5" t="str">
-        <x:v>Cwn Tillery</x:v>
+        <x:v>Abersycan (1887-1889)</x:v>
       </x:c>
       <x:c r="B89" s="5" t="str">
-        <x:v>Cwmtillery</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="C89" s="5" t="str"/>
       <x:c r="D89" s="5" t="str"/>
       <x:c r="E89" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F89" s="5" t="str"/>
+      <x:c r="F89" s="5" t="str">
+        <x:v>1887-1889</x:v>
+      </x:c>
       <x:c r="G89" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H89" s="5" t="str"/>
       <x:c r="I89" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwn_Tillery.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersycan_(1887-1889).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Abersychan (1848-1876)</x:v>
       </x:c>
       <x:c r="B90" s="5" t="str">
-        <x:v>Dinas</x:v>
+        <x:v>Abersychan</x:v>
       </x:c>
       <x:c r="C90" s="5" t="str"/>
       <x:c r="D90" s="5" t="str"/>
       <x:c r="E90" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F90" s="5" t="str"/>
+      <x:c r="F90" s="5" t="str">
+        <x:v>1848-1876</x:v>
+      </x:c>
       <x:c r="G90" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H90" s="5" t="str"/>
       <x:c r="I90" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dinas.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abersychan_(1848-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Abertawe (see Swansea)</x:v>
       </x:c>
       <x:c r="B91" s="5" t="str">
-        <x:v>Dowlais</x:v>
-      </x:c>
-      <x:c r="C91" s="5" t="str"/>
-      <x:c r="D91" s="5" t="str"/>
+        <x:v>Swansea</x:v>
+      </x:c>
+      <x:c r="C91" s="5" t="str">
+        <x:v>Swansea</x:v>
+      </x:c>
+      <x:c r="D91" s="5" t="str">
+        <x:v>See Swansea — possible rename, merger, transfer, or cross-reference; verify before classifying.</x:v>
+      </x:c>
       <x:c r="E91" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
@@ -4735,15 +4785,15 @@
       </x:c>
       <x:c r="H91" s="5" t="str"/>
       <x:c r="I91" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertawe_(see_Swansea).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="5" t="str">
-        <x:v>Dowlais (1851-1872)</x:v>
+        <x:v>Abertillery (1861-1866)</x:v>
       </x:c>
       <x:c r="B92" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Abertillery</x:v>
       </x:c>
       <x:c r="C92" s="5" t="str"/>
       <x:c r="D92" s="5" t="str"/>
@@ -4751,148 +4801,160 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F92" s="5" t="str">
-        <x:v>1851-1872</x:v>
+        <x:v>1861-1866</x:v>
       </x:c>
       <x:c r="G92" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H92" s="5" t="str"/>
       <x:c r="I92" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais_(1851-1872).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Abertillery_(1861-1866).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="5" t="str">
-        <x:v>Ebbro Vale</x:v>
+        <x:v>Alltwen (1849-1859)</x:v>
       </x:c>
       <x:c r="B93" s="5" t="str">
-        <x:v>Ebbw Vale</x:v>
+        <x:v>Alltwen</x:v>
       </x:c>
       <x:c r="C93" s="5" t="str"/>
       <x:c r="D93" s="5" t="str"/>
       <x:c r="E93" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F93" s="5" t="str"/>
+      <x:c r="F93" s="5" t="str">
+        <x:v>1849-1859</x:v>
+      </x:c>
       <x:c r="G93" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H93" s="5" t="str"/>
       <x:c r="I93" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ebbro_Vale.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Alltwen_(1849-1859).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="5" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Brechfa (1846-1868)</x:v>
       </x:c>
       <x:c r="B94" s="5" t="str">
-        <x:v>Ffestiniog</x:v>
+        <x:v>Brechfa</x:v>
       </x:c>
       <x:c r="C94" s="5" t="str"/>
       <x:c r="D94" s="5" t="str"/>
       <x:c r="E94" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F94" s="5" t="str"/>
+      <x:c r="F94" s="5" t="str">
+        <x:v>1846-1868</x:v>
+      </x:c>
       <x:c r="G94" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H94" s="5" t="str"/>
       <x:c r="I94" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ffestiniog.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Brechfa_(1846-1868).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="5" t="str">
-        <x:v>Georgetown</x:v>
+        <x:v>Cardiff (1849-1855)</x:v>
       </x:c>
       <x:c r="B95" s="5" t="str">
-        <x:v>Georgetown</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C95" s="5" t="str"/>
       <x:c r="D95" s="5" t="str"/>
       <x:c r="E95" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F95" s="5" t="str"/>
+      <x:c r="F95" s="5" t="str">
+        <x:v>1849-1855</x:v>
+      </x:c>
       <x:c r="G95" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H95" s="5" t="str"/>
       <x:c r="I95" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Georgetown.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1849-1855).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="5" t="str">
-        <x:v>Gilwern</x:v>
+        <x:v>Cardiff (1854-1876)</x:v>
       </x:c>
       <x:c r="B96" s="5" t="str">
-        <x:v>Gilwern</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C96" s="5" t="str"/>
       <x:c r="D96" s="5" t="str"/>
       <x:c r="E96" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F96" s="5" t="str"/>
+      <x:c r="F96" s="5" t="str">
+        <x:v>1854-1876</x:v>
+      </x:c>
       <x:c r="G96" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H96" s="5" t="str"/>
       <x:c r="I96" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gilwern.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1854-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="5" t="str">
-        <x:v>Gwernllwyn</x:v>
+        <x:v>Cardiff (1931-1947)</x:v>
       </x:c>
       <x:c r="B97" s="5" t="str">
-        <x:v>Dowlais</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C97" s="5" t="str"/>
       <x:c r="D97" s="5" t="str"/>
       <x:c r="E97" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F97" s="5" t="str"/>
+      <x:c r="F97" s="5" t="str">
+        <x:v>1931-1947</x:v>
+      </x:c>
       <x:c r="G97" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H97" s="5" t="str"/>
       <x:c r="I97" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gwernllwyn.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(1931-1947).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Cardiff (Early to 1917, 1919)</x:v>
       </x:c>
       <x:c r="B98" s="5" t="str">
-        <x:v>Haverfordwest</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C98" s="5" t="str"/>
       <x:c r="D98" s="5" t="str"/>
       <x:c r="E98" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F98" s="5" t="str"/>
+      <x:c r="F98" s="5" t="str">
+        <x:v>1917-1919</x:v>
+      </x:c>
       <x:c r="G98" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H98" s="5" t="str"/>
       <x:c r="I98" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Haverfordwest.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_(Early_to_1917,_1919).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Cardiff Branch</x:v>
       </x:c>
       <x:c r="B99" s="5" t="str">
-        <x:v>Llandebie</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C99" s="5" t="str"/>
       <x:c r="D99" s="5" t="str"/>
@@ -4905,59 +4967,59 @@
       </x:c>
       <x:c r="H99" s="5" t="str"/>
       <x:c r="I99" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llandebie.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cardiff_Branch.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="5" t="str">
-        <x:v>Llanelli (1851-1867)</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="B100" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C100" s="5" t="str"/>
       <x:c r="D100" s="5" t="str"/>
       <x:c r="E100" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F100" s="5" t="str">
-        <x:v>1851-1867</x:v>
-      </x:c>
+      <x:c r="F100" s="5" t="str"/>
       <x:c r="G100" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H100" s="5" t="str"/>
       <x:c r="I100" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelli_(1851-1867).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Castell_Nedd_(Neath).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Cefncoed-y-Cymar (1847-1864)</x:v>
       </x:c>
       <x:c r="B101" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="C101" s="5" t="str"/>
       <x:c r="D101" s="5" t="str"/>
       <x:c r="E101" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F101" s="5" t="str"/>
+      <x:c r="F101" s="5" t="str">
+        <x:v>1847-1864</x:v>
+      </x:c>
       <x:c r="G101" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H101" s="5" t="str"/>
       <x:c r="I101" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelltyd.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cefncoed-y-Cymar_(1847-1864).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="5" t="str">
-        <x:v>Llanelly (1847-1849)</x:v>
+        <x:v>Coal Brock Vale (1856-1867)</x:v>
       </x:c>
       <x:c r="B102" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Coalbrookvale</x:v>
       </x:c>
       <x:c r="C102" s="5" t="str"/>
       <x:c r="D102" s="5" t="str"/>
@@ -4965,22 +5027,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F102" s="5" t="str">
-        <x:v>1847-1849</x:v>
+        <x:v>1856-1867</x:v>
       </x:c>
       <x:c r="G102" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H102" s="5" t="str"/>
       <x:c r="I102" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1849).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Coal_Brock_Vale_(1856-1867).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="5" t="str">
-        <x:v>Llanelly (1847-1868)</x:v>
+        <x:v>Cog (1848-1876)</x:v>
       </x:c>
       <x:c r="B103" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="C103" s="5" t="str"/>
       <x:c r="D103" s="5" t="str"/>
@@ -4988,22 +5050,22 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F103" s="5" t="str">
-        <x:v>1847-1868</x:v>
+        <x:v>1848-1876</x:v>
       </x:c>
       <x:c r="G103" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H103" s="5" t="str"/>
       <x:c r="I103" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1868).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cog_(1848-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="5" t="str">
-        <x:v>Llanelly (1857-1863)</x:v>
+        <x:v>Crumlin (1857-1862)</x:v>
       </x:c>
       <x:c r="B104" s="5" t="str">
-        <x:v>Llanelli</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="C104" s="5" t="str"/>
       <x:c r="D104" s="5" t="str"/>
@@ -5011,43 +5073,45 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F104" s="5" t="str">
-        <x:v>1857-1863</x:v>
+        <x:v>1857-1862</x:v>
       </x:c>
       <x:c r="G104" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H104" s="5" t="str"/>
       <x:c r="I104" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1857-1863).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Crumlin_(1857-1862).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="5" t="str">
-        <x:v>Llanelly 2</x:v>
+        <x:v>Cuffern Mountain (1849-1876)</x:v>
       </x:c>
       <x:c r="B105" s="5" t="str">
-        <x:v>Llanelly 2</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="C105" s="5" t="str"/>
       <x:c r="D105" s="5" t="str"/>
       <x:c r="E105" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F105" s="5" t="str"/>
+      <x:c r="F105" s="5" t="str">
+        <x:v>1849-1876</x:v>
+      </x:c>
       <x:c r="G105" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H105" s="5" t="str"/>
       <x:c r="I105" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_2.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cuffern_Mountain_(1849-1876).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Cwm Celin</x:v>
       </x:c>
       <x:c r="B106" s="5" t="str">
-        <x:v>Llanfabon</x:v>
+        <x:v>Cwm Celyn</x:v>
       </x:c>
       <x:c r="C106" s="5" t="str"/>
       <x:c r="D106" s="5" t="str"/>
@@ -5060,15 +5124,15 @@
       </x:c>
       <x:c r="H106" s="5" t="str"/>
       <x:c r="I106" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanfabon.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwm_Celin.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Cwn Tillery</x:v>
       </x:c>
       <x:c r="B107" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Cwmtillery</x:v>
       </x:c>
       <x:c r="C107" s="5" t="str"/>
       <x:c r="D107" s="5" t="str"/>
@@ -5081,61 +5145,57 @@
       </x:c>
       <x:c r="H107" s="5" t="str"/>
       <x:c r="I107" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llansawel.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Cwn_Tillery.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="5" t="str">
-        <x:v>Machen (1854-1865)</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="B108" s="5" t="str">
-        <x:v>Machen</x:v>
+        <x:v>Dinas</x:v>
       </x:c>
       <x:c r="C108" s="5" t="str"/>
       <x:c r="D108" s="5" t="str"/>
       <x:c r="E108" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F108" s="5" t="str">
-        <x:v>1854-1865</x:v>
-      </x:c>
+      <x:c r="F108" s="5" t="str"/>
       <x:c r="G108" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H108" s="5" t="str"/>
       <x:c r="I108" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Machen_(1854-1865).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dinas.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="5" t="str">
-        <x:v>Merthyr Tydfil (1843-1856)</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="B109" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="C109" s="5" t="str"/>
       <x:c r="D109" s="5" t="str"/>
       <x:c r="E109" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F109" s="5" t="str">
-        <x:v>1843-1856</x:v>
-      </x:c>
+      <x:c r="F109" s="5" t="str"/>
       <x:c r="G109" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H109" s="5" t="str"/>
       <x:c r="I109" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1843-1856).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="5" t="str">
-        <x:v>Merthyr Tydfil (1861-1896)</x:v>
+        <x:v>Dowlais (1851-1872)</x:v>
       </x:c>
       <x:c r="B110" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="C110" s="5" t="str"/>
       <x:c r="D110" s="5" t="str"/>
@@ -5143,45 +5203,43 @@
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F110" s="5" t="str">
-        <x:v>1861-1896</x:v>
+        <x:v>1851-1872</x:v>
       </x:c>
       <x:c r="G110" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H110" s="5" t="str"/>
       <x:c r="I110" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1861-1896).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Dowlais_(1851-1872).htm</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="5" t="str">
-        <x:v>Merthyr Tydfil (Early to 1847)</x:v>
+        <x:v>Ebbro Vale</x:v>
       </x:c>
       <x:c r="B111" s="5" t="str">
-        <x:v>Merthyr Tydfil</x:v>
+        <x:v>Ebbw Vale</x:v>
       </x:c>
       <x:c r="C111" s="5" t="str"/>
       <x:c r="D111" s="5" t="str"/>
       <x:c r="E111" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F111" s="5" t="str">
-        <x:v>1847</x:v>
-      </x:c>
+      <x:c r="F111" s="5" t="str"/>
       <x:c r="G111" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H111" s="5" t="str"/>
       <x:c r="I111" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(Early_to_1847).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ebbro_Vale.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="5" t="str">
-        <x:v>Nanty Glo</x:v>
+        <x:v>Ffestiniog</x:v>
       </x:c>
       <x:c r="B112" s="5" t="str">
-        <x:v>Nantyglo</x:v>
+        <x:v>Ffestiniog</x:v>
       </x:c>
       <x:c r="C112" s="5" t="str"/>
       <x:c r="D112" s="5" t="str"/>
@@ -5194,15 +5252,15 @@
       </x:c>
       <x:c r="H112" s="5" t="str"/>
       <x:c r="I112" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Nanty_Glo.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Ffestiniog.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="5" t="str">
-        <x:v>Neath</x:v>
+        <x:v>Georgetown</x:v>
       </x:c>
       <x:c r="B113" s="5" t="str">
-        <x:v>Castell Nedd (Neath)</x:v>
+        <x:v>Georgetown</x:v>
       </x:c>
       <x:c r="C113" s="5" t="str"/>
       <x:c r="D113" s="5" t="str"/>
@@ -5215,498 +5273,480 @@
       </x:c>
       <x:c r="H113" s="5" t="str"/>
       <x:c r="I113" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Neath.htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Georgetown.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="5" t="str">
-        <x:v>Pen-Y-Cae (1844-1866)</x:v>
+        <x:v>Gilwern</x:v>
       </x:c>
       <x:c r="B114" s="5" t="str">
-        <x:v>Pen-y-cae</x:v>
+        <x:v>Gilwern</x:v>
       </x:c>
       <x:c r="C114" s="5" t="str"/>
       <x:c r="D114" s="5" t="str"/>
       <x:c r="E114" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F114" s="5" t="str">
-        <x:v>1844-1866</x:v>
-      </x:c>
+      <x:c r="F114" s="5" t="str"/>
       <x:c r="G114" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H114" s="5" t="str"/>
       <x:c r="I114" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pen-Y-Cae_(1844-1866).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gilwern.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="5" t="str">
-        <x:v>Pontlanfraith (Early to 1947)</x:v>
+        <x:v>Gwernllwyn</x:v>
       </x:c>
       <x:c r="B115" s="5" t="str">
-        <x:v>Pontlanfraith</x:v>
+        <x:v>Dowlais</x:v>
       </x:c>
       <x:c r="C115" s="5" t="str"/>
       <x:c r="D115" s="5" t="str"/>
       <x:c r="E115" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F115" s="5" t="str">
-        <x:v>1947</x:v>
-      </x:c>
+      <x:c r="F115" s="5" t="str"/>
       <x:c r="G115" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H115" s="5" t="str"/>
       <x:c r="I115" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontlanfraith_(Early_to_1947).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Gwernllwyn.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="5" t="str">
-        <x:v>Pontypridd (1877-1895)</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="B116" s="5" t="str">
-        <x:v>Pontypridd</x:v>
+        <x:v>Haverfordwest</x:v>
       </x:c>
       <x:c r="C116" s="5" t="str"/>
       <x:c r="D116" s="5" t="str"/>
       <x:c r="E116" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F116" s="5" t="str">
-        <x:v>1877-1895</x:v>
-      </x:c>
+      <x:c r="F116" s="5" t="str"/>
       <x:c r="G116" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H116" s="5" t="str"/>
       <x:c r="I116" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontypridd_(1877-1895).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Haverfordwest.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="5" t="str">
-        <x:v>Welsh Conference (1850-1922)</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="B117" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Llandebie</x:v>
       </x:c>
       <x:c r="C117" s="5" t="str"/>
       <x:c r="D117" s="5" t="str"/>
       <x:c r="E117" s="5" t="str">
         <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
-      <x:c r="F117" s="5" t="str">
-        <x:v>1850-1922</x:v>
-      </x:c>
+      <x:c r="F117" s="5" t="str"/>
       <x:c r="G117" s="5" t="str">
         <x:v>Wales2Utah research note</x:v>
       </x:c>
       <x:c r="H117" s="5" t="str"/>
       <x:c r="I117" s="5" t="str">
-        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Welsh_Conference_(1850-1922).htm</x:v>
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llandebie.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Llanelli (1851-1867)</x:v>
       </x:c>
       <x:c r="B118" s="5" t="str">
-        <x:v>Cardiff</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C118" s="5" t="str"/>
       <x:c r="D118" s="5" t="str"/>
       <x:c r="E118" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F118" s="5" t="str">
-        <x:v>ca. 1846-1947</x:v>
+        <x:v>1851-1867</x:v>
       </x:c>
       <x:c r="G118" s="5" t="str">
-        <x:v>Film 104168 Items 1-6</x:v>
-      </x:c>
-      <x:c r="H118" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I118" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H118" s="5" t="str"/>
+      <x:c r="I118" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelli_(1851-1867).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="5" t="str">
-        <x:v>Cefncoedycymer</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="B119" s="5" t="str">
-        <x:v>Cefn Coed-y-Cymmer</x:v>
+        <x:v>Llanelltyd</x:v>
       </x:c>
       <x:c r="C119" s="5" t="str"/>
       <x:c r="D119" s="5" t="str"/>
       <x:c r="E119" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F119" s="5" t="str">
-        <x:v>1847-1864</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F119" s="5" t="str"/>
       <x:c r="G119" s="5" t="str">
-        <x:v>Film 104168 Item 7</x:v>
-      </x:c>
-      <x:c r="H119" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I119" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H119" s="5" t="str"/>
+      <x:c r="I119" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelltyd.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="5" t="str">
-        <x:v>Coalbrook Vale</x:v>
+        <x:v>Llanelly (1847-1849)</x:v>
       </x:c>
       <x:c r="B120" s="5" t="str">
-        <x:v>Coalbrookvale</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C120" s="5" t="str"/>
       <x:c r="D120" s="5" t="str"/>
       <x:c r="E120" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F120" s="5" t="str">
-        <x:v>ca. 1856-1867</x:v>
+        <x:v>1847-1849</x:v>
       </x:c>
       <x:c r="G120" s="5" t="str">
-        <x:v>Film 104168 Item 8</x:v>
-      </x:c>
-      <x:c r="H120" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I120" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H120" s="5" t="str"/>
+      <x:c r="I120" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1849).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Llanelly (1847-1868)</x:v>
       </x:c>
       <x:c r="B121" s="5" t="str">
-        <x:v>Cogan</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C121" s="5" t="str"/>
       <x:c r="D121" s="5" t="str"/>
       <x:c r="E121" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F121" s="5" t="str">
-        <x:v>ca. 1848-1876</x:v>
+        <x:v>1847-1868</x:v>
       </x:c>
       <x:c r="G121" s="5" t="str">
-        <x:v>Film 104168 Item 9</x:v>
-      </x:c>
-      <x:c r="H121" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I121" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H121" s="5" t="str"/>
+      <x:c r="I121" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1847-1868).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Llanelly (1857-1863)</x:v>
       </x:c>
       <x:c r="B122" s="5" t="str">
-        <x:v>Crumlin</x:v>
+        <x:v>Llanelli</x:v>
       </x:c>
       <x:c r="C122" s="5" t="str"/>
       <x:c r="D122" s="5" t="str"/>
       <x:c r="E122" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F122" s="5" t="str">
-        <x:v>ca. 1857-1862</x:v>
+        <x:v>1857-1863</x:v>
       </x:c>
       <x:c r="G122" s="5" t="str">
-        <x:v>Film 104168 Item 10</x:v>
-      </x:c>
-      <x:c r="H122" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I122" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H122" s="5" t="str"/>
+      <x:c r="I122" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_(1857-1863).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Llanelly 2</x:v>
       </x:c>
       <x:c r="B123" s="5" t="str">
-        <x:v>Cuffern Mountain</x:v>
+        <x:v>Llanelly 2</x:v>
       </x:c>
       <x:c r="C123" s="5" t="str"/>
       <x:c r="D123" s="5" t="str"/>
       <x:c r="E123" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F123" s="5" t="str">
-        <x:v>1849-1876</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F123" s="5" t="str"/>
       <x:c r="G123" s="5" t="str">
-        <x:v>Film 104168 Item 11</x:v>
-      </x:c>
-      <x:c r="H123" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I123" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H123" s="5" t="str"/>
+      <x:c r="I123" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanelly_2.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="5" t="str">
-        <x:v>Cwmcillyn</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="B124" s="5" t="str">
-        <x:v>Cwmcillyn</x:v>
+        <x:v>Llanfabon</x:v>
       </x:c>
       <x:c r="C124" s="5" t="str"/>
       <x:c r="D124" s="5" t="str"/>
       <x:c r="E124" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F124" s="5" t="str">
-        <x:v>1847-1856</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F124" s="5" t="str"/>
       <x:c r="G124" s="5" t="str">
-        <x:v>Film 104168 Item 12</x:v>
-      </x:c>
-      <x:c r="H124" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I124" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H124" s="5" t="str"/>
+      <x:c r="I124" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Llanfabon.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="5" t="str">
-        <x:v>Cwmbran</x:v>
+        <x:v>Machen (1854-1865)</x:v>
       </x:c>
       <x:c r="B125" s="5" t="str">
-        <x:v>Cwmbran</x:v>
+        <x:v>Machen</x:v>
       </x:c>
       <x:c r="C125" s="5" t="str"/>
       <x:c r="D125" s="5" t="str"/>
       <x:c r="E125" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F125" s="5" t="str">
-        <x:v>1850-1874</x:v>
+        <x:v>1854-1865</x:v>
       </x:c>
       <x:c r="G125" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
-      </x:c>
-      <x:c r="H125" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I125" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H125" s="5" t="str"/>
+      <x:c r="I125" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Machen_(1854-1865).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="5" t="str">
-        <x:v>Llanelltud</x:v>
+        <x:v>Merthyr Tydfil (1843-1856)</x:v>
       </x:c>
       <x:c r="B126" s="5" t="str">
-        <x:v>Llanelltyd</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C126" s="5" t="str"/>
       <x:c r="D126" s="5" t="str"/>
       <x:c r="E126" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F126" s="5" t="str">
-        <x:v>1850-1874</x:v>
+        <x:v>1843-1856</x:v>
       </x:c>
       <x:c r="G126" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
-      </x:c>
-      <x:c r="H126" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I126" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H126" s="5" t="str"/>
+      <x:c r="I126" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1843-1856).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Merthyr Tydfil (1861-1896)</x:v>
       </x:c>
       <x:c r="B127" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C127" s="5" t="str"/>
       <x:c r="D127" s="5" t="str"/>
       <x:c r="E127" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F127" s="5" t="str">
-        <x:v>1875-1882</x:v>
+        <x:v>1861-1896</x:v>
       </x:c>
       <x:c r="G127" s="5" t="str">
-        <x:v>Film 104168 Item 13</x:v>
-      </x:c>
-      <x:c r="H127" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
-      </x:c>
-      <x:c r="I127" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H127" s="5" t="str"/>
+      <x:c r="I127" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(1861-1896).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="5" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Merthyr Tydfil (Early to 1847)</x:v>
       </x:c>
       <x:c r="B128" s="5" t="str">
-        <x:v>Treboeth</x:v>
+        <x:v>Merthyr Tydfil</x:v>
       </x:c>
       <x:c r="C128" s="5" t="str"/>
       <x:c r="D128" s="5" t="str"/>
       <x:c r="E128" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F128" s="5" t="str">
-        <x:v>1844-1880</x:v>
+        <x:v>1847</x:v>
       </x:c>
       <x:c r="G128" s="5" t="str">
-        <x:v>Film 104172 Item 1</x:v>
-      </x:c>
-      <x:c r="H128" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I128" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H128" s="5" t="str"/>
+      <x:c r="I128" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Merthyr_Tydfil_(Early_to_1847).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="5" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Nanty Glo</x:v>
       </x:c>
       <x:c r="B129" s="5" t="str">
-        <x:v>Tredegar</x:v>
+        <x:v>Nantyglo</x:v>
       </x:c>
       <x:c r="C129" s="5" t="str"/>
       <x:c r="D129" s="5" t="str"/>
       <x:c r="E129" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F129" s="5" t="str">
-        <x:v>ca. 1844-1883</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F129" s="5" t="str"/>
       <x:c r="G129" s="5" t="str">
-        <x:v>Film 104172 Items 2-3</x:v>
-      </x:c>
-      <x:c r="H129" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I129" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H129" s="5" t="str"/>
+      <x:c r="I129" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Nanty_Glo.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="5" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Neath</x:v>
       </x:c>
       <x:c r="B130" s="5" t="str">
-        <x:v>Treforest</x:v>
+        <x:v>Castell Nedd (Neath)</x:v>
       </x:c>
       <x:c r="C130" s="5" t="str"/>
       <x:c r="D130" s="5" t="str"/>
       <x:c r="E130" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
-      </x:c>
-      <x:c r="F130" s="5" t="str">
-        <x:v>1851-1873</x:v>
-      </x:c>
+        <x:v>Recovered RoboHelp branch note</x:v>
+      </x:c>
+      <x:c r="F130" s="5" t="str"/>
       <x:c r="G130" s="5" t="str">
-        <x:v>Film 104172 Item 4</x:v>
-      </x:c>
-      <x:c r="H130" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I130" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H130" s="5" t="str"/>
+      <x:c r="I130" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Neath.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="5" t="str">
-        <x:v>Morriston</x:v>
+        <x:v>Pen-Y-Cae (1844-1866)</x:v>
       </x:c>
       <x:c r="B131" s="5" t="str">
-        <x:v>Morriston</x:v>
+        <x:v>Pen-y-cae</x:v>
       </x:c>
       <x:c r="C131" s="5" t="str"/>
       <x:c r="D131" s="5" t="str"/>
       <x:c r="E131" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F131" s="5" t="str">
-        <x:v>1853-1868</x:v>
+        <x:v>1844-1866</x:v>
       </x:c>
       <x:c r="G131" s="5" t="str">
-        <x:v>Film 104172 Item 5</x:v>
-      </x:c>
-      <x:c r="H131" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I131" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H131" s="5" t="str"/>
+      <x:c r="I131" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pen-Y-Cae_(1844-1866).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Pontlanfraith (Early to 1947)</x:v>
       </x:c>
       <x:c r="B132" s="5" t="str">
-        <x:v>Treorchy</x:v>
+        <x:v>Pontlanfraith</x:v>
       </x:c>
       <x:c r="C132" s="5" t="str"/>
       <x:c r="D132" s="5" t="str"/>
       <x:c r="E132" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F132" s="5" t="str">
-        <x:v>1875-1882</x:v>
+        <x:v>1947</x:v>
       </x:c>
       <x:c r="G132" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
-      </x:c>
-      <x:c r="H132" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I132" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H132" s="5" t="str"/>
+      <x:c r="I132" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontlanfraith_(Early_to_1947).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="5" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Pontypridd (1877-1895)</x:v>
       </x:c>
       <x:c r="B133" s="5" t="str">
-        <x:v>Trinant</x:v>
+        <x:v>Pontypridd</x:v>
       </x:c>
       <x:c r="C133" s="5" t="str"/>
       <x:c r="D133" s="5" t="str"/>
       <x:c r="E133" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F133" s="5" t="str">
-        <x:v>ca. 1849-1853</x:v>
+        <x:v>1877-1895</x:v>
       </x:c>
       <x:c r="G133" s="5" t="str">
-        <x:v>Film 104172 Item 6</x:v>
-      </x:c>
-      <x:c r="H133" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I133" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H133" s="5" t="str"/>
+      <x:c r="I133" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Pontypridd_(1877-1895).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Welsh Conference (1850-1922)</x:v>
       </x:c>
       <x:c r="B134" s="5" t="str">
-        <x:v>Rhymney English</x:v>
+        <x:v>Welsh Conference</x:v>
       </x:c>
       <x:c r="C134" s="5" t="str"/>
       <x:c r="D134" s="5" t="str"/>
       <x:c r="E134" s="5" t="str">
-        <x:v>FamilySearch catalog</x:v>
+        <x:v>Recovered RoboHelp branch note</x:v>
       </x:c>
       <x:c r="F134" s="5" t="str">
-        <x:v>1851-1883</x:v>
+        <x:v>1850-1922</x:v>
       </x:c>
       <x:c r="G134" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
-      </x:c>
-      <x:c r="H134" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
-      </x:c>
-      <x:c r="I134" s="5" t="str"/>
+        <x:v>Wales2Utah research note</x:v>
+      </x:c>
+      <x:c r="H134" s="5" t="str"/>
+      <x:c r="I134" s="5" t="str">
+        <x:v>C:\Users\kenro\Desktop\HOME\RH\RH_OUTPUT\Wales2Utah_RawBranches\LDS\Branches\Welsh_Conference_(1850-1922).htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="5" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="B135" s="5" t="str">
-        <x:v>Twyncarno</x:v>
+        <x:v>Cardiff</x:v>
       </x:c>
       <x:c r="C135" s="5" t="str"/>
       <x:c r="D135" s="5" t="str"/>
@@ -5714,22 +5754,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F135" s="5" t="str">
-        <x:v>1851-1883</x:v>
+        <x:v>ca. 1846-1947</x:v>
       </x:c>
       <x:c r="G135" s="5" t="str">
-        <x:v>Film 104172 Items 7-8</x:v>
+        <x:v>Film 104168 Items 1-6</x:v>
       </x:c>
       <x:c r="H135" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I135" s="5" t="str"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="5" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Cefncoedycymer</x:v>
       </x:c>
       <x:c r="B136" s="5" t="str">
-        <x:v>Twyn-yr-Odyn</x:v>
+        <x:v>Cefn Coed-y-Cymmer</x:v>
       </x:c>
       <x:c r="C136" s="5" t="str"/>
       <x:c r="D136" s="5" t="str"/>
@@ -5737,22 +5777,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F136" s="5" t="str">
-        <x:v>1847-1901</x:v>
+        <x:v>1847-1864</x:v>
       </x:c>
       <x:c r="G136" s="5" t="str">
-        <x:v>Film 104172 Items 9-10</x:v>
+        <x:v>Film 104168 Item 7</x:v>
       </x:c>
       <x:c r="H136" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I136" s="5" t="str"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Coalbrook Vale</x:v>
       </x:c>
       <x:c r="B137" s="5" t="str">
-        <x:v>Welsh Conference</x:v>
+        <x:v>Coalbrookvale</x:v>
       </x:c>
       <x:c r="C137" s="5" t="str"/>
       <x:c r="D137" s="5" t="str"/>
@@ -5760,22 +5800,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F137" s="5" t="str">
-        <x:v>ca. 1850-1922</x:v>
+        <x:v>ca. 1856-1867</x:v>
       </x:c>
       <x:c r="G137" s="5" t="str">
-        <x:v>Film 104172 Item 11</x:v>
+        <x:v>Film 104168 Item 8</x:v>
       </x:c>
       <x:c r="H137" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I137" s="5" t="str"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="5" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="B138" s="5" t="str">
-        <x:v>Ystrad</x:v>
+        <x:v>Cogan</x:v>
       </x:c>
       <x:c r="C138" s="5" t="str"/>
       <x:c r="D138" s="5" t="str"/>
@@ -5783,22 +5823,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F138" s="5" t="str">
-        <x:v>ca. 1885-1911</x:v>
+        <x:v>ca. 1848-1876</x:v>
       </x:c>
       <x:c r="G138" s="5" t="str">
-        <x:v>Film 104172 Item 12</x:v>
+        <x:v>Film 104168 Item 9</x:v>
       </x:c>
       <x:c r="H138" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I138" s="5" t="str"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="B139" s="5" t="str">
-        <x:v>Llansawel</x:v>
+        <x:v>Crumlin</x:v>
       </x:c>
       <x:c r="C139" s="5" t="str"/>
       <x:c r="D139" s="5" t="str"/>
@@ -5806,22 +5846,22 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F139" s="5" t="str">
-        <x:v>1849-1855; 1850-1853; 1879</x:v>
+        <x:v>ca. 1857-1862</x:v>
       </x:c>
       <x:c r="G139" s="5" t="str">
-        <x:v>Film 104169 items 14-15</x:v>
+        <x:v>Film 104168 Item 10</x:v>
       </x:c>
       <x:c r="H139" s="5" t="str">
-        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
       </x:c>
       <x:c r="I139" s="5" t="str"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="B140" s="5" t="str">
-        <x:v>Sutton Mountain</x:v>
+        <x:v>Cuffern Mountain</x:v>
       </x:c>
       <x:c r="C140" s="5" t="str"/>
       <x:c r="D140" s="5" t="str"/>
@@ -5829,20 +5869,480 @@
         <x:v>FamilySearch catalog</x:v>
       </x:c>
       <x:c r="F140" s="5" t="str">
+        <x:v>1849-1876</x:v>
+      </x:c>
+      <x:c r="G140" s="5" t="str">
+        <x:v>Film 104168 Item 11</x:v>
+      </x:c>
+      <x:c r="H140" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
+      <x:c r="I140" s="5" t="str"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="5" t="str">
+        <x:v>Cwmcillyn</x:v>
+      </x:c>
+      <x:c r="B141" s="5" t="str">
+        <x:v>Cwmcillyn</x:v>
+      </x:c>
+      <x:c r="C141" s="5" t="str"/>
+      <x:c r="D141" s="5" t="str"/>
+      <x:c r="E141" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F141" s="5" t="str">
+        <x:v>1847-1856</x:v>
+      </x:c>
+      <x:c r="G141" s="5" t="str">
+        <x:v>Film 104168 Item 12</x:v>
+      </x:c>
+      <x:c r="H141" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
+      <x:c r="I141" s="5" t="str"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="5" t="str">
+        <x:v>Cwmbran</x:v>
+      </x:c>
+      <x:c r="B142" s="5" t="str">
+        <x:v>Cwmbran</x:v>
+      </x:c>
+      <x:c r="C142" s="5" t="str"/>
+      <x:c r="D142" s="5" t="str"/>
+      <x:c r="E142" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F142" s="5" t="str">
+        <x:v>1850-1874</x:v>
+      </x:c>
+      <x:c r="G142" s="5" t="str">
+        <x:v>Film 104168 Item 13</x:v>
+      </x:c>
+      <x:c r="H142" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
+      <x:c r="I142" s="5" t="str"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="5" t="str">
+        <x:v>Llanelltud</x:v>
+      </x:c>
+      <x:c r="B143" s="5" t="str">
+        <x:v>Llanelltyd</x:v>
+      </x:c>
+      <x:c r="C143" s="5" t="str"/>
+      <x:c r="D143" s="5" t="str"/>
+      <x:c r="E143" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F143" s="5" t="str">
+        <x:v>1850-1874</x:v>
+      </x:c>
+      <x:c r="G143" s="5" t="str">
+        <x:v>Film 104168 Item 13</x:v>
+      </x:c>
+      <x:c r="H143" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
+      <x:c r="I143" s="5" t="str"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="5" t="str">
+        <x:v>Treorchy</x:v>
+      </x:c>
+      <x:c r="B144" s="5" t="str">
+        <x:v>Treorchy</x:v>
+      </x:c>
+      <x:c r="C144" s="5" t="str"/>
+      <x:c r="D144" s="5" t="str"/>
+      <x:c r="E144" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F144" s="5" t="str">
+        <x:v>1875-1882</x:v>
+      </x:c>
+      <x:c r="G144" s="5" t="str">
+        <x:v>Film 104168 Item 13</x:v>
+      </x:c>
+      <x:c r="H144" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104168</x:v>
+      </x:c>
+      <x:c r="I144" s="5" t="str"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="5" t="str">
+        <x:v>Treboeth</x:v>
+      </x:c>
+      <x:c r="B145" s="5" t="str">
+        <x:v>Treboeth</x:v>
+      </x:c>
+      <x:c r="C145" s="5" t="str"/>
+      <x:c r="D145" s="5" t="str"/>
+      <x:c r="E145" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F145" s="5" t="str">
+        <x:v>1844-1880</x:v>
+      </x:c>
+      <x:c r="G145" s="5" t="str">
+        <x:v>Film 104172 Item 1</x:v>
+      </x:c>
+      <x:c r="H145" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I145" s="5" t="str"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="5" t="str">
+        <x:v>Tredegar</x:v>
+      </x:c>
+      <x:c r="B146" s="5" t="str">
+        <x:v>Tredegar</x:v>
+      </x:c>
+      <x:c r="C146" s="5" t="str"/>
+      <x:c r="D146" s="5" t="str"/>
+      <x:c r="E146" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F146" s="5" t="str">
+        <x:v>ca. 1844-1883</x:v>
+      </x:c>
+      <x:c r="G146" s="5" t="str">
+        <x:v>Film 104172 Items 2-3</x:v>
+      </x:c>
+      <x:c r="H146" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I146" s="5" t="str"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="5" t="str">
+        <x:v>Treforest</x:v>
+      </x:c>
+      <x:c r="B147" s="5" t="str">
+        <x:v>Treforest</x:v>
+      </x:c>
+      <x:c r="C147" s="5" t="str"/>
+      <x:c r="D147" s="5" t="str"/>
+      <x:c r="E147" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F147" s="5" t="str">
+        <x:v>1851-1873</x:v>
+      </x:c>
+      <x:c r="G147" s="5" t="str">
+        <x:v>Film 104172 Item 4</x:v>
+      </x:c>
+      <x:c r="H147" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I147" s="5" t="str"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="5" t="str">
+        <x:v>Morriston</x:v>
+      </x:c>
+      <x:c r="B148" s="5" t="str">
+        <x:v>Morriston</x:v>
+      </x:c>
+      <x:c r="C148" s="5" t="str"/>
+      <x:c r="D148" s="5" t="str"/>
+      <x:c r="E148" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F148" s="5" t="str">
+        <x:v>1853-1868</x:v>
+      </x:c>
+      <x:c r="G148" s="5" t="str">
+        <x:v>Film 104172 Item 5</x:v>
+      </x:c>
+      <x:c r="H148" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I148" s="5" t="str"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="5" t="str">
+        <x:v>Treorchy</x:v>
+      </x:c>
+      <x:c r="B149" s="5" t="str">
+        <x:v>Treorchy</x:v>
+      </x:c>
+      <x:c r="C149" s="5" t="str"/>
+      <x:c r="D149" s="5" t="str"/>
+      <x:c r="E149" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F149" s="5" t="str">
+        <x:v>1875-1882</x:v>
+      </x:c>
+      <x:c r="G149" s="5" t="str">
+        <x:v>Film 104172 Item 6</x:v>
+      </x:c>
+      <x:c r="H149" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I149" s="5" t="str"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="5" t="str">
+        <x:v>Trinant</x:v>
+      </x:c>
+      <x:c r="B150" s="5" t="str">
+        <x:v>Trinant</x:v>
+      </x:c>
+      <x:c r="C150" s="5" t="str"/>
+      <x:c r="D150" s="5" t="str"/>
+      <x:c r="E150" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F150" s="5" t="str">
+        <x:v>ca. 1849-1853</x:v>
+      </x:c>
+      <x:c r="G150" s="5" t="str">
+        <x:v>Film 104172 Item 6</x:v>
+      </x:c>
+      <x:c r="H150" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I150" s="5" t="str"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="5" t="str">
+        <x:v>Rhymney English</x:v>
+      </x:c>
+      <x:c r="B151" s="5" t="str">
+        <x:v>Rhymney English</x:v>
+      </x:c>
+      <x:c r="C151" s="5" t="str"/>
+      <x:c r="D151" s="5" t="str"/>
+      <x:c r="E151" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F151" s="5" t="str">
+        <x:v>1851-1883</x:v>
+      </x:c>
+      <x:c r="G151" s="5" t="str">
+        <x:v>Film 104172 Items 7-8</x:v>
+      </x:c>
+      <x:c r="H151" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I151" s="5" t="str"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="5" t="str">
+        <x:v>Twyncarno</x:v>
+      </x:c>
+      <x:c r="B152" s="5" t="str">
+        <x:v>Twyncarno</x:v>
+      </x:c>
+      <x:c r="C152" s="5" t="str"/>
+      <x:c r="D152" s="5" t="str"/>
+      <x:c r="E152" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F152" s="5" t="str">
+        <x:v>1851-1883</x:v>
+      </x:c>
+      <x:c r="G152" s="5" t="str">
+        <x:v>Film 104172 Items 7-8</x:v>
+      </x:c>
+      <x:c r="H152" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I152" s="5" t="str"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="5" t="str">
+        <x:v>Twyn-yr-Odyn</x:v>
+      </x:c>
+      <x:c r="B153" s="5" t="str">
+        <x:v>Twyn-yr-Odyn</x:v>
+      </x:c>
+      <x:c r="C153" s="5" t="str"/>
+      <x:c r="D153" s="5" t="str"/>
+      <x:c r="E153" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F153" s="5" t="str">
+        <x:v>1847-1901</x:v>
+      </x:c>
+      <x:c r="G153" s="5" t="str">
+        <x:v>Film 104172 Items 9-10</x:v>
+      </x:c>
+      <x:c r="H153" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I153" s="5" t="str"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="5" t="str">
+        <x:v>Welsh Conference</x:v>
+      </x:c>
+      <x:c r="B154" s="5" t="str">
+        <x:v>Welsh Conference</x:v>
+      </x:c>
+      <x:c r="C154" s="5" t="str"/>
+      <x:c r="D154" s="5" t="str"/>
+      <x:c r="E154" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F154" s="5" t="str">
+        <x:v>ca. 1850-1922</x:v>
+      </x:c>
+      <x:c r="G154" s="5" t="str">
+        <x:v>Film 104172 Item 11</x:v>
+      </x:c>
+      <x:c r="H154" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I154" s="5" t="str"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="5" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="B155" s="5" t="str">
+        <x:v>Ystrad</x:v>
+      </x:c>
+      <x:c r="C155" s="5" t="str"/>
+      <x:c r="D155" s="5" t="str"/>
+      <x:c r="E155" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F155" s="5" t="str">
+        <x:v>ca. 1885-1911</x:v>
+      </x:c>
+      <x:c r="G155" s="5" t="str">
+        <x:v>Film 104172 Item 12</x:v>
+      </x:c>
+      <x:c r="H155" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104172</x:v>
+      </x:c>
+      <x:c r="I155" s="5" t="str"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="5" t="str">
+        <x:v>Llansawel (Carmarthenshire)</x:v>
+      </x:c>
+      <x:c r="B156" s="5" t="str">
+        <x:v>Llansawel (Carmarthenshire)</x:v>
+      </x:c>
+      <x:c r="C156" s="5" t="str"/>
+      <x:c r="D156" s="5" t="str"/>
+      <x:c r="E156" s="5" t="str">
+        <x:v>FamilySearch catalog context</x:v>
+      </x:c>
+      <x:c r="F156" s="5" t="str">
+        <x:v>1849-1855</x:v>
+      </x:c>
+      <x:c r="G156" s="5" t="str">
+        <x:v>Film 104169 items 14-15; locality assignment requires the recovered CD 14 source</x:v>
+      </x:c>
+      <x:c r="H156" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+      </x:c>
+      <x:c r="I156" s="5" t="str"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="5" t="str">
+        <x:v>Llansawel (Glamorgan)</x:v>
+      </x:c>
+      <x:c r="B157" s="5" t="str">
+        <x:v>Llansawel (Glamorgan)</x:v>
+      </x:c>
+      <x:c r="C157" s="5" t="str"/>
+      <x:c r="D157" s="5" t="str"/>
+      <x:c r="E157" s="5" t="str">
+        <x:v>FamilySearch catalog context</x:v>
+      </x:c>
+      <x:c r="F157" s="5" t="str">
+        <x:v>1850-1889</x:v>
+      </x:c>
+      <x:c r="G157" s="5" t="str">
+        <x:v>Film 104169 items 14-15; locality assignment requires the recovered LR 11759 7 heading</x:v>
+      </x:c>
+      <x:c r="H157" s="5" t="str">
+        <x:v>https://www.familysearch.org/search/catalog/209087</x:v>
+      </x:c>
+      <x:c r="I157" s="5" t="str"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="5" t="str">
+        <x:v>Sutton Mountain</x:v>
+      </x:c>
+      <x:c r="B158" s="5" t="str">
+        <x:v>Sutton Mountain</x:v>
+      </x:c>
+      <x:c r="C158" s="5" t="str"/>
+      <x:c r="D158" s="5" t="str"/>
+      <x:c r="E158" s="5" t="str">
+        <x:v>FamilySearch catalog</x:v>
+      </x:c>
+      <x:c r="F158" s="5" t="str">
         <x:v>1853-1859</x:v>
       </x:c>
-      <x:c r="G140" s="5" t="str">
+      <x:c r="G158" s="5" t="str">
         <x:v>Film 104171 item 6</x:v>
       </x:c>
-      <x:c r="H140" s="5" t="str">
+      <x:c r="H158" s="5" t="str">
         <x:v>https://www.familysearch.org/search/catalog/results?query=film_number%3A104171</x:v>
       </x:c>
-      <x:c r="I140" s="5" t="str"/>
+      <x:c r="I158" s="5" t="str"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="5" t="str">
+        <x:v>Cwmbran</x:v>
+      </x:c>
+      <x:c r="B159" s="5" t="str">
+        <x:v>Cwmbran</x:v>
+      </x:c>
+      <x:c r="C159" s="5" t="str"/>
+      <x:c r="D159" s="5" t="str"/>
+      <x:c r="E159" s="5" t="str">
+        <x:v>Typed contextual minutes evidence</x:v>
+      </x:c>
+      <x:c r="F159" s="5" t="str">
+        <x:v>1850-1874</x:v>
+      </x:c>
+      <x:c r="G159" s="5" t="str">
+        <x:v>CD 62 within source group CDs 60-62; LR 70861 1; Pontypool/Abersychan General Minutes, 1857-1889; Cwmbran reports on typed PDF pages 129, 167, 169, 171-172, 176</x:v>
+      </x:c>
+      <x:c r="H159" s="5" t="str"/>
+      <x:c r="I159" s="5" t="str">
+        <x:v>resources/transcriptions/A - CDs 60-62 - Typed Transcripts.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="5" t="str">
+        <x:v>Morriston</x:v>
+      </x:c>
+      <x:c r="B160" s="5" t="str">
+        <x:v>Morriston</x:v>
+      </x:c>
+      <x:c r="C160" s="5" t="str"/>
+      <x:c r="D160" s="5" t="str"/>
+      <x:c r="E160" s="5" t="str">
+        <x:v>Typed contextual minutes evidence</x:v>
+      </x:c>
+      <x:c r="F160" s="5" t="str">
+        <x:v>1853-1868</x:v>
+      </x:c>
+      <x:c r="G160" s="5" t="str">
+        <x:v>CD 41; LR 17617 21; Western Glamorgan Conference Minutes, 1851-1870; Morriston fast-offerings report, 1866</x:v>
+      </x:c>
+      <x:c r="H160" s="5" t="str"/>
+      <x:c r="I160" s="5" t="str">
+        <x:v>resources/transcriptions/A - CDs 40-43 (2 of 2) - Typed Transcripts.pdf</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R130e0acf4c4b443d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R013fb85279db499d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>